<commit_message>
test upload for cloud run
</commit_message>
<xml_diff>
--- a/outputs/contracts_analysis.xlsx
+++ b/outputs/contracts_analysis.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -475,12 +475,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>f5efbbfc-fdfb-42f7-9232-a2f3be3daf9f</t>
+          <t>a03b9893-2aed-468c-9c73-ec05cb0384e7</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>pdf_one.pdf</t>
+          <t>pdf_onetwothree.pdf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -493,24 +493,28 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>groq_analysis</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
+          <t>mock_analysis</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>contracts/a03b9893-2aed-468c-9c73-ec05cb0384e7_pdf_onetwothree.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>a4407809-50ad-47e0-a018-f491675eea34</t>
+          <t>cb3658a6-a277-46b9-9024-0172a372e7fe</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>sample_contract.pdf</t>
+          <t>pdf_onetwo.pdf</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -523,24 +527,28 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>mock_analysis</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>contracts/cb3658a6-a277-46b9-9024-0172a372e7fe_pdf_onetwo.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>b78e24be-a635-465b-bbf2-528df3030ebe</t>
+          <t>d75be996-aa63-4afa-b444-43028cd8f100</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>file-sample_100kB.doc</t>
+          <t>pdf_onetwo.pdf</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -553,24 +561,28 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>mock_analysis</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
+          <t>groq_analysis</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>contracts/d75be996-aa63-4afa-b444-43028cd8f100_pdf_onetwo.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>02322ecf-25a1-4fa0-8ec3-8170732b158b</t>
+          <t>21f4e271-b4ad-4f99-a14a-94ce47e36526</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>sample_contract.pdf</t>
+          <t>pdf_one.pdf</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -583,24 +595,28 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>mock_analysis</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
+          <t>groq_analysis</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>contracts/21f4e271-b4ad-4f99-a14a-94ce47e36526_pdf_one.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>a4a4156e-13d5-4287-b21b-312a8cf8f963</t>
+          <t>eb66af10-afcd-49b6-9bda-2c9a98104b0d</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>file-sample_100kB.doc</t>
+          <t>pdf_one.pdf</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -613,24 +629,28 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>mock_analysis</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
+          <t>groq_analysis</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>contracts/eb66af10-afcd-49b6-9bda-2c9a98104b0d_pdf_one.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>9d53d74b-da2a-4072-8402-890806ece509</t>
+          <t>6e2af0ae-e9c2-4704-a033-3f15c315f9ee</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>sample_contract.pdf</t>
+          <t>pdf_one.pdf</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -643,11 +663,11 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>mock_analysis</t>
+          <t>groq_analysis</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -655,12 +675,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>f5d109b6-8bdf-4364-bfa0-8d10c795291f</t>
+          <t>760dae3f-2e15-452d-b26d-b6e0f0d61455</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>file-sample_100kB.doc</t>
+          <t>pdf_one.pdf</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -673,11 +693,11 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>mock_analysis</t>
+          <t>groq_analysis</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
@@ -685,12 +705,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>6882dc89-ec45-480e-9b40-68026dc5b421</t>
+          <t>75be4ed5-c26d-4f1b-bcae-b7459f580ab2</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>sample_contract.pdf</t>
+          <t>pdf_one.pdf</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -703,11 +723,11 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>mock_analysis</t>
+          <t>groq_analysis</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -715,12 +735,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>df910248-91c5-45a6-b3d2-deb8d52c50e2</t>
+          <t>ae2be41f-5311-41ff-a26a-30d0ddd76b83</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>file-sample_100kB.doc</t>
+          <t>pdf_one.pdf</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -733,11 +753,11 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>mock_analysis</t>
+          <t>groq_analysis</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -745,12 +765,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>7f84a4f8-5947-4a69-9a74-08393b2a8c73</t>
+          <t>b2093736-d821-46c9-89b3-c0df20783f68</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>sample_contract.pdf</t>
+          <t>pdf_one.pdf</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -763,11 +783,11 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>mock_analysis</t>
+          <t>groq_analysis</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -775,12 +795,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>643394d8-6cae-42fd-b536-12046f1056d9</t>
+          <t>125ca547-322f-4c26-89a1-b4a255ceade3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>file-sample_100kB.doc</t>
+          <t>pdf_one.pdf</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -793,11 +813,11 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>mock_analysis</t>
+          <t>groq_analysis</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -805,12 +825,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04bf9fd3-6cd0-4a73-a15e-ad4fc525ae8d</t>
+          <t>f5efbbfc-fdfb-42f7-9232-a2f3be3daf9f</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>sample_contract.pdf</t>
+          <t>pdf_one.pdf</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -823,11 +843,11 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>mock_analysis</t>
+          <t>groq_analysis</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -835,12 +855,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>cbf7f90a-4c4a-4844-ac98-c9c970fdaf57</t>
+          <t>a4407809-50ad-47e0-a018-f491675eea34</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>file-sample_100kB.doc</t>
+          <t>sample_contract.pdf</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -853,14 +873,344 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
+        <v>100</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>mock_analysis</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>b78e24be-a635-465b-bbf2-528df3030ebe</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>file-sample_100kB.doc</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>contract</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="n">
         <v>60</v>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>mock_analysis</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>02322ecf-25a1-4fa0-8ec3-8170732b158b</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>sample_contract.pdf</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>contract</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>100</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>mock_analysis</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>a4a4156e-13d5-4287-b21b-312a8cf8f963</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>file-sample_100kB.doc</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>contract</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>60</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>mock_analysis</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>9d53d74b-da2a-4072-8402-890806ece509</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>sample_contract.pdf</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>contract</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="n">
+        <v>100</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>mock_analysis</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>f5d109b6-8bdf-4364-bfa0-8d10c795291f</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>file-sample_100kB.doc</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>contract</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>60</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>mock_analysis</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>6882dc89-ec45-480e-9b40-68026dc5b421</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>sample_contract.pdf</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>contract</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>100</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>mock_analysis</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>df910248-91c5-45a6-b3d2-deb8d52c50e2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>file-sample_100kB.doc</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>contract</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>60</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>mock_analysis</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>7f84a4f8-5947-4a69-9a74-08393b2a8c73</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>sample_contract.pdf</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>contract</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="n">
+        <v>100</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>mock_analysis</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>643394d8-6cae-42fd-b536-12046f1056d9</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>file-sample_100kB.doc</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>contract</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="n">
+        <v>60</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>mock_analysis</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>04bf9fd3-6cd0-4a73-a15e-ad4fc525ae8d</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>sample_contract.pdf</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>contract</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="n">
+        <v>100</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>mock_analysis</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>cbf7f90a-4c4a-4844-ac98-c9c970fdaf57</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>file-sample_100kB.doc</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>contract</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="n">
+        <v>60</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>mock_analysis</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -886,7 +1236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -914,78 +1264,292 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>f5efbbfc-fdfb-42f7-9232-a2f3be3daf9f</t>
+          <t>a03b9893-2aed-468c-9c73-ec05cb0384e7</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>pdf_one.pdf</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
+          <t>pdf_onetwothree.pdf</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Governing Law</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Governing Law: Delaware.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>a4407809-50ad-47e0-a018-f491675eea34</t>
+          <t>a03b9893-2aed-468c-9c73-ec05cb0384e7</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>sample_contract.pdf</t>
+          <t>pdf_onetwothree.pdf</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Termination</t>
+          <t>Liability</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Termination Clause: Either party may terminate with 30 days written notice.</t>
+          <t>The vendor shall indemnify the customer without any liability cap.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>a4407809-50ad-47e0-a018-f491675eea34</t>
+          <t>cb3658a6-a277-46b9-9024-0172a372e7fe</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>sample_contract.pdf</t>
+          <t>pdf_onetwo.pdf</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Confidentiality</t>
+          <t>Governing Law</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Confidentiality Clause: Both parties agree to keep confidential information private.</t>
+          <t>Governing Law: Delaware.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>cb3658a6-a277-46b9-9024-0172a372e7fe</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>pdf_onetwo.pdf</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Liability</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>The vendor shall indemnify the customer without any liability cap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>d75be996-aa63-4afa-b444-43028cd8f100</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>pdf_onetwo.pdf</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>21f4e271-b4ad-4f99-a14a-94ce47e36526</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>eb66af10-afcd-49b6-9bda-2c9a98104b0d</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>6e2af0ae-e9c2-4704-a033-3f15c315f9ee</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>760dae3f-2e15-452d-b26d-b6e0f0d61455</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>75be4ed5-c26d-4f1b-bcae-b7459f580ab2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ae2be41f-5311-41ff-a26a-30d0ddd76b83</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>b2093736-d821-46c9-89b3-c0df20783f68</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>125ca547-322f-4c26-89a1-b4a255ceade3</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>f5efbbfc-fdfb-42f7-9232-a2f3be3daf9f</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>a4407809-50ad-47e0-a018-f491675eea34</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Termination</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Termination Clause: Either party may terminate with 30 days written notice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>a4407809-50ad-47e0-a018-f491675eea34</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>sample_contract.pdf</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Confidentiality</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Confidentiality Clause: Both parties agree to keep confidential information private.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>a4407809-50ad-47e0-a018-f491675eea34</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>sample_contract.pdf</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
         <is>
           <t>Payment</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Effective Date: January 1, 2025
 Expiration Date: December 31, 2025
@@ -993,89 +1557,89 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>a4407809-50ad-47e0-a018-f491675eea34</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Governing Law</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Governing Law: State of California.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>02322ecf-25a1-4fa0-8ec3-8170732b158b</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Termination</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Termination Clause: Either party may terminate with 30 days written notice.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>02322ecf-25a1-4fa0-8ec3-8170732b158b</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Confidentiality</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Confidentiality Clause: Both parties agree to keep confidential information private.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>02322ecf-25a1-4fa0-8ec3-8170732b158b</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Payment</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Effective Date: January 1, 2025
 Expiration Date: December 31, 2025
@@ -1083,89 +1647,89 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>02322ecf-25a1-4fa0-8ec3-8170732b158b</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Governing Law</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Governing Law: State of California.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>9d53d74b-da2a-4072-8402-890806ece509</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Termination</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Termination Clause: Either party may terminate with 30 days written notice.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>9d53d74b-da2a-4072-8402-890806ece509</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>Confidentiality</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Confidentiality Clause: Both parties agree to keep confidential information private.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>9d53d74b-da2a-4072-8402-890806ece509</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Payment</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>Effective Date: January 1, 2025
 Expiration Date: December 31, 2025
@@ -1173,89 +1737,89 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>9d53d74b-da2a-4072-8402-890806ece509</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Governing Law</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Governing Law: State of California.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>6882dc89-ec45-480e-9b40-68026dc5b421</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Termination</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>Termination Clause: Either party may terminate with 30 days written notice.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>6882dc89-ec45-480e-9b40-68026dc5b421</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Confidentiality</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Confidentiality Clause: Both parties agree to keep confidential information private.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>6882dc89-ec45-480e-9b40-68026dc5b421</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Payment</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>Effective Date: January 1, 2025
 Expiration Date: December 31, 2025
@@ -1263,89 +1827,89 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>6882dc89-ec45-480e-9b40-68026dc5b421</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>Governing Law</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>Governing Law: State of California.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>7f84a4f8-5947-4a69-9a74-08393b2a8c73</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>Termination</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Termination Clause: Either party may terminate with 30 days written notice.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>7f84a4f8-5947-4a69-9a74-08393b2a8c73</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>Confidentiality</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>Confidentiality Clause: Both parties agree to keep confidential information private.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>7f84a4f8-5947-4a69-9a74-08393b2a8c73</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>Payment</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Effective Date: January 1, 2025
 Expiration Date: December 31, 2025
@@ -1353,89 +1917,89 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>7f84a4f8-5947-4a69-9a74-08393b2a8c73</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>Governing Law</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>Governing Law: State of California.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>04bf9fd3-6cd0-4a73-a15e-ad4fc525ae8d</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>Termination</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>Termination Clause: Either party may terminate with 30 days written notice.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>04bf9fd3-6cd0-4a73-a15e-ad4fc525ae8d</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>Confidentiality</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>Confidentiality Clause: Both parties agree to keep confidential information private.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t>04bf9fd3-6cd0-4a73-a15e-ad4fc525ae8d</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>Payment</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>Effective Date: January 1, 2025
 Expiration Date: December 31, 2025
@@ -1443,23 +2007,23 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>04bf9fd3-6cd0-4a73-a15e-ad4fc525ae8d</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>Governing Law</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>Governing Law: State of California.</t>
         </is>
@@ -1476,7 +2040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1509,27 +2073,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>f5efbbfc-fdfb-42f7-9232-a2f3be3daf9f</t>
+          <t>a03b9893-2aed-468c-9c73-ec05cb0384e7</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>pdf_one.pdf</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+          <t>pdf_onetwothree.pdf</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Termination clause may be missing</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>No termination keyword found.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>b78e24be-a635-465b-bbf2-528df3030ebe</t>
+          <t>cb3658a6-a277-46b9-9024-0172a372e7fe</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>file-sample_100kB.doc</t>
+          <t>pdf_onetwo.pdf</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1551,295 +2127,472 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>b78e24be-a635-465b-bbf2-528df3030ebe</t>
+          <t>d75be996-aa63-4afa-b444-43028cd8f100</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>file-sample_100kB.doc</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Governing law clause may be missing</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>No governing law keyword found.</t>
-        </is>
-      </c>
+          <t>pdf_onetwo.pdf</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>a4a4156e-13d5-4287-b21b-312a8cf8f963</t>
+          <t>21f4e271-b4ad-4f99-a14a-94ce47e36526</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>file-sample_100kB.doc</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Termination clause may be missing</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>No termination keyword found.</t>
-        </is>
-      </c>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>a4a4156e-13d5-4287-b21b-312a8cf8f963</t>
+          <t>eb66af10-afcd-49b6-9bda-2c9a98104b0d</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>file-sample_100kB.doc</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Governing law clause may be missing</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>No governing law keyword found.</t>
-        </is>
-      </c>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>f5d109b6-8bdf-4364-bfa0-8d10c795291f</t>
+          <t>6e2af0ae-e9c2-4704-a033-3f15c315f9ee</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>file-sample_100kB.doc</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Termination clause may be missing</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>No termination keyword found.</t>
-        </is>
-      </c>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>f5d109b6-8bdf-4364-bfa0-8d10c795291f</t>
+          <t>760dae3f-2e15-452d-b26d-b6e0f0d61455</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>file-sample_100kB.doc</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Governing law clause may be missing</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>No governing law keyword found.</t>
-        </is>
-      </c>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>df910248-91c5-45a6-b3d2-deb8d52c50e2</t>
+          <t>75be4ed5-c26d-4f1b-bcae-b7459f580ab2</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>file-sample_100kB.doc</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Termination clause may be missing</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>No termination keyword found.</t>
-        </is>
-      </c>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>df910248-91c5-45a6-b3d2-deb8d52c50e2</t>
+          <t>ae2be41f-5311-41ff-a26a-30d0ddd76b83</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>file-sample_100kB.doc</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Governing law clause may be missing</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>No governing law keyword found.</t>
-        </is>
-      </c>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>643394d8-6cae-42fd-b536-12046f1056d9</t>
+          <t>b2093736-d821-46c9-89b3-c0df20783f68</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>file-sample_100kB.doc</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Termination clause may be missing</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>No termination keyword found.</t>
-        </is>
-      </c>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>643394d8-6cae-42fd-b536-12046f1056d9</t>
+          <t>125ca547-322f-4c26-89a1-b4a255ceade3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>file-sample_100kB.doc</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Governing law clause may be missing</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>No governing law keyword found.</t>
-        </is>
-      </c>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>cbf7f90a-4c4a-4844-ac98-c9c970fdaf57</t>
+          <t>f5efbbfc-fdfb-42f7-9232-a2f3be3daf9f</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>file-sample_100kB.doc</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Termination clause may be missing</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>No termination keyword found.</t>
-        </is>
-      </c>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>b78e24be-a635-465b-bbf2-528df3030ebe</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>file-sample_100kB.doc</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Termination clause may be missing</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>No termination keyword found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>b78e24be-a635-465b-bbf2-528df3030ebe</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>file-sample_100kB.doc</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Governing law clause may be missing</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>No governing law keyword found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>a4a4156e-13d5-4287-b21b-312a8cf8f963</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>file-sample_100kB.doc</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Termination clause may be missing</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>No termination keyword found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>a4a4156e-13d5-4287-b21b-312a8cf8f963</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>file-sample_100kB.doc</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Governing law clause may be missing</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>No governing law keyword found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>f5d109b6-8bdf-4364-bfa0-8d10c795291f</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>file-sample_100kB.doc</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Termination clause may be missing</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>No termination keyword found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>f5d109b6-8bdf-4364-bfa0-8d10c795291f</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>file-sample_100kB.doc</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Governing law clause may be missing</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>No governing law keyword found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>df910248-91c5-45a6-b3d2-deb8d52c50e2</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>file-sample_100kB.doc</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Termination clause may be missing</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>No termination keyword found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>df910248-91c5-45a6-b3d2-deb8d52c50e2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>file-sample_100kB.doc</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Governing law clause may be missing</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>No governing law keyword found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>643394d8-6cae-42fd-b536-12046f1056d9</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>file-sample_100kB.doc</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Termination clause may be missing</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>No termination keyword found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>643394d8-6cae-42fd-b536-12046f1056d9</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>file-sample_100kB.doc</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Governing law clause may be missing</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>No governing law keyword found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>cbf7f90a-4c4a-4844-ac98-c9c970fdaf57</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>file-sample_100kB.doc</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Termination clause may be missing</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>No termination keyword found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>cbf7f90a-4c4a-4844-ac98-c9c970fdaf57</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>file-sample_100kB.doc</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
         <is>
           <t>Governing law clause may be missing</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>No governing law keyword found.</t>
         </is>
@@ -1856,7 +2609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1879,15 +2632,309 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>f5efbbfc-fdfb-42f7-9232-a2f3be3daf9f</t>
+          <t>a03b9893-2aed-468c-9c73-ec05cb0384e7</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>pdf_one.pdf</t>
+          <t>pdf_onetwothree.pdf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
+        <is>
+          <t>--- Page 1 ---
+This Agreement is made between Alpha Technologies and Beta Solutio
+Effective Date: June 20, 2026.
+Term: 12 months.
+Governing Law: Delaware.
+The agreement automatically renews for one year unless either party g
+Either party may terminate with 90 days notice.
+The vendor shall indemnify the customer without any liability cap.
+--- Page 2 ---
+Lorem ipsum 
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. Nunc ac faucibus odio. 
+Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut
+varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum
+condimentum.  Vivamus  dapibus  sodales  ex,  vitae  malesuada  ipsum  cursus
+convallis. Maecenas sed egestas nulla, ac condimentum orci.  Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus.
+
+Maecenas non lorem quis tellus placerat varius. 
+
+Nulla facilisi. 
+
+Aenean congue fringilla justo ut aliquam. 
+
+Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante
+sagittis. 
+
+Morbi viverra semper lorem nec molestie. 
+
+Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+Row 1
+Row 2
+Row 3
+Row 4
+0
+2
+4
+6
+8
+10
+12
+Column 1
+Column 2
+Column 3
+--- Page 3 ---
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. Fusce vitae vestibulum velit. Pellentesque
+vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas
+velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci
+maximus ultricies. 
+Cras fringilla ipsum magna, in fringilla dui commodo 
+a.
+Lorem ipsum
+Lorem ipsum
+Lorem ipsum
+1
+In eleifend velit vitae libero sollicitudin euismod.
+Lorem
+2
+Cras fringilla ipsum magna, in fringilla dui commodo
+a.
+Ipsum
+3
+Aliquam erat volutpat. 
+Lorem
+4
+Fusce vitae vestibulum velit. 
+Lorem
+5
+Etiam vehicula luctus fermentum.
+Ipsum
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 4 ---
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. 
+Nunc ac faucibus odio. Vestibulum neque massa, scelerisque sit amet ligula eu, congue
+molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor
+vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum
+cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit 
+dictum tellus. 
+Maecenas non lorem quis tellus placerat varius. Nulla facilisi. Aenean congue fringilla justo
+ut aliquam. Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum
+ante sagittis. Morbi viverra semper lorem nec molestie. Maecenas tincidunt est efficitur
+ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. 
+Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo.
+Aliquam  erat volutpat.  Vestibulum  in  egestas  velit. Pellentesque  fermentum nisl  vitae
+fringilla  venenatis.  Etiam  id  mauris  vitae  orci  maximus  ultricies.  Cras  fringilla  ipsum
+magna, in fringilla dui commodo a.
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 5 ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>cb3658a6-a277-46b9-9024-0172a372e7fe</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>pdf_onetwo.pdf</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>--- Page 1 ---
+This Agreement is made between Alpha Technologies and Beta Solutio
+Effective Date: June 20, 2026.
+Term: 12 months.
+Governing Law: Delaware.
+The agreement automatically renews for one year unless either party g
+Either party may terminate with 90 days notice.
+The vendor shall indemnify the customer without any liability cap.
+--- Page 2 ---
+Lorem ipsum 
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. Nunc ac faucibus odio. 
+Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut
+varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum
+condimentum.  Vivamus  dapibus  sodales  ex,  vitae  malesuada  ipsum  cursus
+convallis. Maecenas sed egestas nulla, ac condimentum orci.  Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus.
+
+Maecenas non lorem quis tellus placerat varius. 
+
+Nulla facilisi. 
+
+Aenean congue fringilla justo ut aliquam. 
+
+Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante
+sagittis. 
+
+Morbi viverra semper lorem nec molestie. 
+
+Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+Row 1
+Row 2
+Row 3
+Row 4
+0
+2
+4
+6
+8
+10
+12
+Column 1
+Column 2
+Column 3
+--- Page 3 ---
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. Fusce vitae vestibulum velit. Pellentesque
+vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas
+velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci
+maximus ultricies. 
+Cras fringilla ipsum magna, in fringilla dui commodo 
+a.
+Lorem ipsum
+Lorem ipsum
+Lorem ipsum
+1
+In eleifend velit vitae libero sollicitudin euismod.
+Lorem
+2
+Cras fringilla ipsum magna, in fringilla dui commodo
+a.
+Ipsum
+3
+Aliquam erat volutpat. 
+Lorem
+4
+Fusce vitae vestibulum velit. 
+Lorem
+5
+Etiam vehicula luctus fermentum.
+Ipsum
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 4 ---
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. 
+Nunc ac faucibus odio. Vestibulum neque massa, scelerisque sit amet ligula eu, congue
+molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor
+vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum
+cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit 
+dictum tellus. 
+Maecenas non lorem quis tellus placerat varius. Nulla facilisi. Aenean congue fringilla justo
+ut aliquam. Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum
+ante sagittis. Morbi viverra semper lorem nec molestie. Maecenas tincidunt est efficitur
+ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. 
+Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo.
+Aliquam  erat volutpat.  Vestibulum  in  egestas  velit. Pellentesque  fermentum nisl  vitae
+fringilla  venenatis.  Etiam  id  mauris  vitae  orci  maximus  ultricies.  Cras  fringilla  ipsum
+magna, in fringilla dui commodo a.
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 5 ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>d75be996-aa63-4afa-b444-43028cd8f100</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>pdf_onetwo.pdf</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
         <is>
           <t>--- Page 1 ---
 Lorem ipsum 
@@ -2015,18 +3062,1269 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>21f4e271-b4ad-4f99-a14a-94ce47e36526</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>--- Page 1 ---
+Lorem ipsum 
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. Nunc ac faucibus odio. 
+Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut
+varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum
+condimentum.  Vivamus  dapibus  sodales  ex,  vitae  malesuada  ipsum  cursus
+convallis. Maecenas sed egestas nulla, ac condimentum orci.  Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus.
+
+Maecenas non lorem quis tellus placerat varius. 
+
+Nulla facilisi. 
+
+Aenean congue fringilla justo ut aliquam. 
+
+Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante
+sagittis. 
+
+Morbi viverra semper lorem nec molestie. 
+
+Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+Row 1
+Row 2
+Row 3
+Row 4
+0
+2
+4
+6
+8
+10
+12
+Column 1
+Column 2
+Column 3
+--- Page 2 ---
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. Fusce vitae vestibulum velit. Pellentesque
+vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas
+velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci
+maximus ultricies. 
+Cras fringilla ipsum magna, in fringilla dui commodo 
+a.
+Lorem ipsum
+Lorem ipsum
+Lorem ipsum
+1
+In eleifend velit vitae libero sollicitudin euismod.
+Lorem
+2
+Cras fringilla ipsum magna, in fringilla dui commodo
+a.
+Ipsum
+3
+Aliquam erat volutpat. 
+Lorem
+4
+Fusce vitae vestibulum velit. 
+Lorem
+5
+Etiam vehicula luctus fermentum.
+Ipsum
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 3 ---
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. 
+Nunc ac faucibus odio. Vestibulum neque massa, scelerisque sit amet ligula eu, congue
+molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor
+vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum
+cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit 
+dictum tellus. 
+Maecenas non lorem quis tellus placerat varius. Nulla facilisi. Aenean congue fringilla justo
+ut aliquam. Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum
+ante sagittis. Morbi viverra semper lorem nec molestie. Maecenas tincidunt est efficitur
+ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. 
+Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo.
+Aliquam  erat volutpat.  Vestibulum  in  egestas  velit. Pellentesque  fermentum nisl  vitae
+fringilla  venenatis.  Etiam  id  mauris  vitae  orci  maximus  ultricies.  Cras  fringilla  ipsum
+magna, in fringilla dui commodo a.
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 4 ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>eb66af10-afcd-49b6-9bda-2c9a98104b0d</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>--- Page 1 ---
+Lorem ipsum 
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. Nunc ac faucibus odio. 
+Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut
+varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum
+condimentum.  Vivamus  dapibus  sodales  ex,  vitae  malesuada  ipsum  cursus
+convallis. Maecenas sed egestas nulla, ac condimentum orci.  Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus.
+
+Maecenas non lorem quis tellus placerat varius. 
+
+Nulla facilisi. 
+
+Aenean congue fringilla justo ut aliquam. 
+
+Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante
+sagittis. 
+
+Morbi viverra semper lorem nec molestie. 
+
+Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+Row 1
+Row 2
+Row 3
+Row 4
+0
+2
+4
+6
+8
+10
+12
+Column 1
+Column 2
+Column 3
+--- Page 2 ---
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. Fusce vitae vestibulum velit. Pellentesque
+vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas
+velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci
+maximus ultricies. 
+Cras fringilla ipsum magna, in fringilla dui commodo 
+a.
+Lorem ipsum
+Lorem ipsum
+Lorem ipsum
+1
+In eleifend velit vitae libero sollicitudin euismod.
+Lorem
+2
+Cras fringilla ipsum magna, in fringilla dui commodo
+a.
+Ipsum
+3
+Aliquam erat volutpat. 
+Lorem
+4
+Fusce vitae vestibulum velit. 
+Lorem
+5
+Etiam vehicula luctus fermentum.
+Ipsum
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 3 ---
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. 
+Nunc ac faucibus odio. Vestibulum neque massa, scelerisque sit amet ligula eu, congue
+molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor
+vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum
+cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit 
+dictum tellus. 
+Maecenas non lorem quis tellus placerat varius. Nulla facilisi. Aenean congue fringilla justo
+ut aliquam. Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum
+ante sagittis. Morbi viverra semper lorem nec molestie. Maecenas tincidunt est efficitur
+ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. 
+Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo.
+Aliquam  erat volutpat.  Vestibulum  in  egestas  velit. Pellentesque  fermentum nisl  vitae
+fringilla  venenatis.  Etiam  id  mauris  vitae  orci  maximus  ultricies.  Cras  fringilla  ipsum
+magna, in fringilla dui commodo a.
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 4 ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>6e2af0ae-e9c2-4704-a033-3f15c315f9ee</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>--- Page 1 ---
+Lorem ipsum 
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. Nunc ac faucibus odio. 
+Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut
+varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum
+condimentum.  Vivamus  dapibus  sodales  ex,  vitae  malesuada  ipsum  cursus
+convallis. Maecenas sed egestas nulla, ac condimentum orci.  Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus.
+
+Maecenas non lorem quis tellus placerat varius. 
+
+Nulla facilisi. 
+
+Aenean congue fringilla justo ut aliquam. 
+
+Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante
+sagittis. 
+
+Morbi viverra semper lorem nec molestie. 
+
+Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+Row 1
+Row 2
+Row 3
+Row 4
+0
+2
+4
+6
+8
+10
+12
+Column 1
+Column 2
+Column 3
+--- Page 2 ---
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. Fusce vitae vestibulum velit. Pellentesque
+vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas
+velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci
+maximus ultricies. 
+Cras fringilla ipsum magna, in fringilla dui commodo 
+a.
+Lorem ipsum
+Lorem ipsum
+Lorem ipsum
+1
+In eleifend velit vitae libero sollicitudin euismod.
+Lorem
+2
+Cras fringilla ipsum magna, in fringilla dui commodo
+a.
+Ipsum
+3
+Aliquam erat volutpat. 
+Lorem
+4
+Fusce vitae vestibulum velit. 
+Lorem
+5
+Etiam vehicula luctus fermentum.
+Ipsum
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 3 ---
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. 
+Nunc ac faucibus odio. Vestibulum neque massa, scelerisque sit amet ligula eu, congue
+molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor
+vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum
+cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit 
+dictum tellus. 
+Maecenas non lorem quis tellus placerat varius. Nulla facilisi. Aenean congue fringilla justo
+ut aliquam. Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum
+ante sagittis. Morbi viverra semper lorem nec molestie. Maecenas tincidunt est efficitur
+ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. 
+Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo.
+Aliquam  erat volutpat.  Vestibulum  in  egestas  velit. Pellentesque  fermentum nisl  vitae
+fringilla  venenatis.  Etiam  id  mauris  vitae  orci  maximus  ultricies.  Cras  fringilla  ipsum
+magna, in fringilla dui commodo a.
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 4 ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>760dae3f-2e15-452d-b26d-b6e0f0d61455</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>--- Page 1 ---
+Lorem ipsum 
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. Nunc ac faucibus odio. 
+Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut
+varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum
+condimentum.  Vivamus  dapibus  sodales  ex,  vitae  malesuada  ipsum  cursus
+convallis. Maecenas sed egestas nulla, ac condimentum orci.  Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus.
+
+Maecenas non lorem quis tellus placerat varius. 
+
+Nulla facilisi. 
+
+Aenean congue fringilla justo ut aliquam. 
+
+Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante
+sagittis. 
+
+Morbi viverra semper lorem nec molestie. 
+
+Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+Row 1
+Row 2
+Row 3
+Row 4
+0
+2
+4
+6
+8
+10
+12
+Column 1
+Column 2
+Column 3
+--- Page 2 ---
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. Fusce vitae vestibulum velit. Pellentesque
+vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas
+velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci
+maximus ultricies. 
+Cras fringilla ipsum magna, in fringilla dui commodo 
+a.
+Lorem ipsum
+Lorem ipsum
+Lorem ipsum
+1
+In eleifend velit vitae libero sollicitudin euismod.
+Lorem
+2
+Cras fringilla ipsum magna, in fringilla dui commodo
+a.
+Ipsum
+3
+Aliquam erat volutpat. 
+Lorem
+4
+Fusce vitae vestibulum velit. 
+Lorem
+5
+Etiam vehicula luctus fermentum.
+Ipsum
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 3 ---
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. 
+Nunc ac faucibus odio. Vestibulum neque massa, scelerisque sit amet ligula eu, congue
+molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor
+vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum
+cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit 
+dictum tellus. 
+Maecenas non lorem quis tellus placerat varius. Nulla facilisi. Aenean congue fringilla justo
+ut aliquam. Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum
+ante sagittis. Morbi viverra semper lorem nec molestie. Maecenas tincidunt est efficitur
+ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. 
+Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo.
+Aliquam  erat volutpat.  Vestibulum  in  egestas  velit. Pellentesque  fermentum nisl  vitae
+fringilla  venenatis.  Etiam  id  mauris  vitae  orci  maximus  ultricies.  Cras  fringilla  ipsum
+magna, in fringilla dui commodo a.
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 4 ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>75be4ed5-c26d-4f1b-bcae-b7459f580ab2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>--- Page 1 ---
+Lorem ipsum 
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. Nunc ac faucibus odio. 
+Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut
+varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum
+condimentum.  Vivamus  dapibus  sodales  ex,  vitae  malesuada  ipsum  cursus
+convallis. Maecenas sed egestas nulla, ac condimentum orci.  Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus.
+
+Maecenas non lorem quis tellus placerat varius. 
+
+Nulla facilisi. 
+
+Aenean congue fringilla justo ut aliquam. 
+
+Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante
+sagittis. 
+
+Morbi viverra semper lorem nec molestie. 
+
+Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+Row 1
+Row 2
+Row 3
+Row 4
+0
+2
+4
+6
+8
+10
+12
+Column 1
+Column 2
+Column 3
+--- Page 2 ---
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. Fusce vitae vestibulum velit. Pellentesque
+vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas
+velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci
+maximus ultricies. 
+Cras fringilla ipsum magna, in fringilla dui commodo 
+a.
+Lorem ipsum
+Lorem ipsum
+Lorem ipsum
+1
+In eleifend velit vitae libero sollicitudin euismod.
+Lorem
+2
+Cras fringilla ipsum magna, in fringilla dui commodo
+a.
+Ipsum
+3
+Aliquam erat volutpat. 
+Lorem
+4
+Fusce vitae vestibulum velit. 
+Lorem
+5
+Etiam vehicula luctus fermentum.
+Ipsum
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 3 ---
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. 
+Nunc ac faucibus odio. Vestibulum neque massa, scelerisque sit amet ligula eu, congue
+molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor
+vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum
+cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit 
+dictum tellus. 
+Maecenas non lorem quis tellus placerat varius. Nulla facilisi. Aenean congue fringilla justo
+ut aliquam. Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum
+ante sagittis. Morbi viverra semper lorem nec molestie. Maecenas tincidunt est efficitur
+ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. 
+Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo.
+Aliquam  erat volutpat.  Vestibulum  in  egestas  velit. Pellentesque  fermentum nisl  vitae
+fringilla  venenatis.  Etiam  id  mauris  vitae  orci  maximus  ultricies.  Cras  fringilla  ipsum
+magna, in fringilla dui commodo a.
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 4 ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ae2be41f-5311-41ff-a26a-30d0ddd76b83</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>--- Page 1 ---
+Lorem ipsum 
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. Nunc ac faucibus odio. 
+Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut
+varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum
+condimentum.  Vivamus  dapibus  sodales  ex,  vitae  malesuada  ipsum  cursus
+convallis. Maecenas sed egestas nulla, ac condimentum orci.  Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus.
+
+Maecenas non lorem quis tellus placerat varius. 
+
+Nulla facilisi. 
+
+Aenean congue fringilla justo ut aliquam. 
+
+Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante
+sagittis. 
+
+Morbi viverra semper lorem nec molestie. 
+
+Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+Row 1
+Row 2
+Row 3
+Row 4
+0
+2
+4
+6
+8
+10
+12
+Column 1
+Column 2
+Column 3
+--- Page 2 ---
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. Fusce vitae vestibulum velit. Pellentesque
+vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas
+velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci
+maximus ultricies. 
+Cras fringilla ipsum magna, in fringilla dui commodo 
+a.
+Lorem ipsum
+Lorem ipsum
+Lorem ipsum
+1
+In eleifend velit vitae libero sollicitudin euismod.
+Lorem
+2
+Cras fringilla ipsum magna, in fringilla dui commodo
+a.
+Ipsum
+3
+Aliquam erat volutpat. 
+Lorem
+4
+Fusce vitae vestibulum velit. 
+Lorem
+5
+Etiam vehicula luctus fermentum.
+Ipsum
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 3 ---
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. 
+Nunc ac faucibus odio. Vestibulum neque massa, scelerisque sit amet ligula eu, congue
+molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor
+vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum
+cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit 
+dictum tellus. 
+Maecenas non lorem quis tellus placerat varius. Nulla facilisi. Aenean congue fringilla justo
+ut aliquam. Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum
+ante sagittis. Morbi viverra semper lorem nec molestie. Maecenas tincidunt est efficitur
+ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. 
+Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo.
+Aliquam  erat volutpat.  Vestibulum  in  egestas  velit. Pellentesque  fermentum nisl  vitae
+fringilla  venenatis.  Etiam  id  mauris  vitae  orci  maximus  ultricies.  Cras  fringilla  ipsum
+magna, in fringilla dui commodo a.
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 4 ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>b2093736-d821-46c9-89b3-c0df20783f68</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>--- Page 1 ---
+Lorem ipsum 
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. Nunc ac faucibus odio. 
+Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut
+varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum
+condimentum.  Vivamus  dapibus  sodales  ex,  vitae  malesuada  ipsum  cursus
+convallis. Maecenas sed egestas nulla, ac condimentum orci.  Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus.
+
+Maecenas non lorem quis tellus placerat varius. 
+
+Nulla facilisi. 
+
+Aenean congue fringilla justo ut aliquam. 
+
+Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante
+sagittis. 
+
+Morbi viverra semper lorem nec molestie. 
+
+Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+Row 1
+Row 2
+Row 3
+Row 4
+0
+2
+4
+6
+8
+10
+12
+Column 1
+Column 2
+Column 3
+--- Page 2 ---
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. Fusce vitae vestibulum velit. Pellentesque
+vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas
+velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci
+maximus ultricies. 
+Cras fringilla ipsum magna, in fringilla dui commodo 
+a.
+Lorem ipsum
+Lorem ipsum
+Lorem ipsum
+1
+In eleifend velit vitae libero sollicitudin euismod.
+Lorem
+2
+Cras fringilla ipsum magna, in fringilla dui commodo
+a.
+Ipsum
+3
+Aliquam erat volutpat. 
+Lorem
+4
+Fusce vitae vestibulum velit. 
+Lorem
+5
+Etiam vehicula luctus fermentum.
+Ipsum
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 3 ---
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. 
+Nunc ac faucibus odio. Vestibulum neque massa, scelerisque sit amet ligula eu, congue
+molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor
+vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum
+cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit 
+dictum tellus. 
+Maecenas non lorem quis tellus placerat varius. Nulla facilisi. Aenean congue fringilla justo
+ut aliquam. Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum
+ante sagittis. Morbi viverra semper lorem nec molestie. Maecenas tincidunt est efficitur
+ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. 
+Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo.
+Aliquam  erat volutpat.  Vestibulum  in  egestas  velit. Pellentesque  fermentum nisl  vitae
+fringilla  venenatis.  Etiam  id  mauris  vitae  orci  maximus  ultricies.  Cras  fringilla  ipsum
+magna, in fringilla dui commodo a.
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 4 ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>125ca547-322f-4c26-89a1-b4a255ceade3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>--- Page 1 ---
+Lorem ipsum 
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. Nunc ac faucibus odio. 
+Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut
+varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum
+condimentum.  Vivamus  dapibus  sodales  ex,  vitae  malesuada  ipsum  cursus
+convallis. Maecenas sed egestas nulla, ac condimentum orci.  Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus.
+
+Maecenas non lorem quis tellus placerat varius. 
+
+Nulla facilisi. 
+
+Aenean congue fringilla justo ut aliquam. 
+
+Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante
+sagittis. 
+
+Morbi viverra semper lorem nec molestie. 
+
+Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+Row 1
+Row 2
+Row 3
+Row 4
+0
+2
+4
+6
+8
+10
+12
+Column 1
+Column 2
+Column 3
+--- Page 2 ---
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. Fusce vitae vestibulum velit. Pellentesque
+vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas
+velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci
+maximus ultricies. 
+Cras fringilla ipsum magna, in fringilla dui commodo 
+a.
+Lorem ipsum
+Lorem ipsum
+Lorem ipsum
+1
+In eleifend velit vitae libero sollicitudin euismod.
+Lorem
+2
+Cras fringilla ipsum magna, in fringilla dui commodo
+a.
+Ipsum
+3
+Aliquam erat volutpat. 
+Lorem
+4
+Fusce vitae vestibulum velit. 
+Lorem
+5
+Etiam vehicula luctus fermentum.
+Ipsum
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 3 ---
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. 
+Nunc ac faucibus odio. Vestibulum neque massa, scelerisque sit amet ligula eu, congue
+molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor
+vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum
+cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit 
+dictum tellus. 
+Maecenas non lorem quis tellus placerat varius. Nulla facilisi. Aenean congue fringilla justo
+ut aliquam. Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum
+ante sagittis. Morbi viverra semper lorem nec molestie. Maecenas tincidunt est efficitur
+ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. 
+Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo.
+Aliquam  erat volutpat.  Vestibulum  in  egestas  velit. Pellentesque  fermentum nisl  vitae
+fringilla  venenatis.  Etiam  id  mauris  vitae  orci  maximus  ultricies.  Cras  fringilla  ipsum
+magna, in fringilla dui commodo a.
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 4 ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>f5efbbfc-fdfb-42f7-9232-a2f3be3daf9f</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>pdf_one.pdf</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>--- Page 1 ---
+Lorem ipsum 
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. Nunc ac faucibus odio. 
+Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut
+varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum
+condimentum.  Vivamus  dapibus  sodales  ex,  vitae  malesuada  ipsum  cursus
+convallis. Maecenas sed egestas nulla, ac condimentum orci.  Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus.
+
+Maecenas non lorem quis tellus placerat varius. 
+
+Nulla facilisi. 
+
+Aenean congue fringilla justo ut aliquam. 
+
+Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante
+sagittis. 
+
+Morbi viverra semper lorem nec molestie. 
+
+Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+Row 1
+Row 2
+Row 3
+Row 4
+0
+2
+4
+6
+8
+10
+12
+Column 1
+Column 2
+Column 3
+--- Page 2 ---
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. Fusce vitae vestibulum velit. Pellentesque
+vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas
+velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci
+maximus ultricies. 
+Cras fringilla ipsum magna, in fringilla dui commodo 
+a.
+Lorem ipsum
+Lorem ipsum
+Lorem ipsum
+1
+In eleifend velit vitae libero sollicitudin euismod.
+Lorem
+2
+Cras fringilla ipsum magna, in fringilla dui commodo
+a.
+Ipsum
+3
+Aliquam erat volutpat. 
+Lorem
+4
+Fusce vitae vestibulum velit. 
+Lorem
+5
+Etiam vehicula luctus fermentum.
+Ipsum
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 3 ---
+Lorem ipsum dolor sit amet, consectetur adipiscing 
+elit. 
+Nunc ac faucibus odio. Vestibulum neque massa, scelerisque sit amet ligula eu, congue
+molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor
+vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum
+cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis,
+vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus
+nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum,
+ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet
+tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet
+mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit 
+dictum tellus. 
+Maecenas non lorem quis tellus placerat varius. Nulla facilisi. Aenean congue fringilla justo
+ut aliquam. Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum
+ante sagittis. Morbi viverra semper lorem nec molestie. Maecenas tincidunt est efficitur
+ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam
+est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat
+et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis
+tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque
+scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam
+lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel,
+ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. 
+Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo.
+Aliquam  erat volutpat.  Vestibulum  in  egestas  velit. Pellentesque  fermentum nisl  vitae
+fringilla  venenatis.  Etiam  id  mauris  vitae  orci  maximus  ultricies.  Cras  fringilla  ipsum
+magna, in fringilla dui commodo a.
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui.
+Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam,
+pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti
+sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper
+justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo
+posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut
+et  pulvinar  nunc.  Pellentesque  fringilla  mollis  efficitur.  Nullam  venenatis  commodo
+imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem
+sed turpis imperdiet eleifend sit amet id sapien.
+--- Page 4 ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>a4407809-50ad-47e0-a018-f491675eea34</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>--- Page 1 ---
 Sample Service Agreement
@@ -2040,135 +4338,794 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>b78e24be-a635-465b-bbf2-528df3030ebe</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>file-sample_100kB.doc</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ࡱ;		
+ !"#$%&amp;'()*+,-./0123456789:;&lt;=&gt;?@ABCDEFGHIJKLMNOPQRSTUVWXYZ[\]^_`abcdefghijklmnopqrstuvwxyz{|}~Root Entry	
+ !"#$%&amp;'()*+,-./0123456789:;&lt;=&gt;?@ABCE
+	FMicrosoft Word-Dokument
+MSWordDocWord.Document.89qDyKyKNhttps://products.office.com/en-us/wordOh+'0
+px	
+[ZZNormal1$*$3B*OJQJCJmH	sH	KHPJnHtH^JaJ_H9N!2N	Heading 1@&amp;
+&amp;F
+&amp;FxCJ$5aJ$\N!2N	Heading 2@&amp;
+&amp;F
+&amp;FxCJ 5aJ \X!2X	Heading 3@&amp;
+&amp;F
+&amp;FxB*phCJ5aJ\..BulletsOJQJPJ^JJUJ
+Internet Link B*	phmHsH&gt;*nHtH_HZVZVisited Internet Link B*
+phmHsH&gt;*nHtH_HF2FHeading
+x$OJ	QJ	CJPJ^JaJ4B24	Text Bodyd  /1B List^J
+@"R@Caption
+xx$CJ6^J
+aJ]&amp;b&amp;Index$^J
+&lt;r&lt;
+Quotations^7]7`2&gt;!22Title$a$CJ85aJ8\:J!2:Subtitle$a$&lt;xCJ$aJ$44Table Contents$*+*+P9^rD+ 9 !"#$%&amp;'%9dX%'+:X"$D)M Ww v$PR$V:c;1U@|(	
+NA?C"
+NA?C"&lt;
+Cb:r V
+T%(T^`P^`^8`08^`^X`X^`^x`x^``^`^`OJQJ^J^8`8OJQJ^J%^`OJQJ^J%^`OJQJ^J^p`pOJQJ^J%^	`	OJQJ^J%^@`@OJQJ^J^`OJQJ^J%^`OJQJ^J%P
+GTimes New Roman5Symbol3&amp;ArialiLiberation SerifTimes New Roman?&amp;DejaVu SansG
+Open SansArialODroid Sans Fallback9FreeSans_OpenSymbolArial Unicode MSS&amp;Liberation SansArial9$FreeSans5Symbol_OpenSymbolArial Unicode MSBhXg((((' 0 0
+0@@@B.o@
+
+;OBq*sLibreOffice.ChartDocument.1Embedded Object},[PKYKl((mimetypeapplication/vnd.oasis.openM 	0 9Caolan80	aNd+	FFLB
+!b-@6F8 :,~
+!Lorem ipsum 
+Lorem ipsum dolor sit amet, consectetur adipiscing elit. Nunc ac faucibus odio. 
+Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis, vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum, ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus.
+Maecenas non lorem quis tellus placerat varius. 
+Nulla facilisi. 
+Aenean congue fringilla justo ut aliquam. 
+ HYPERLINK "https://products.office.com/en-us/word"Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante sagittis. 
+Morbi viverra semper lorem nec molestie. 
+Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel, ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci maximus ultricies. 
+Cras fringilla ipsum magna, in fringilla dui commodo a.
+Lorem ipsumLorem ipsumLorem ipsum1In eleifend velit vitae libero sollicitudin euismod.Lorem2Cras fringilla ipsum magna, in fringilla dui commodo a.Ipsum3Aliquam erat volutpat. Lorem4Fusce vitae vestibulum velit. Lorem5Etiam vehicula luctus fermentum.Ipsum
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui. Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam, pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut et pulvinar nunc. Pellentesque fringilla mollis efficitur. Nullam venenatis commodo imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem sed turpis imperdiet eleifend sit amet id sapien.
+Lorem ipsum dolor sit amet, consectetur adipiscing elit. 
+Nunc ac faucibus odio. Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis, vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum, ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus. 
+Maecenas non lorem quis tellus placerat varius. Nulla facilisi. Aenean congue fringilla justo ut aliquam. Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante sagittis. Morbi viverra semper lorem nec molestie. Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel, ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. 
+Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci maximus ultricies. Cras fringilla ipsum magna, in fringilla dui commodo a.
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui. Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam, pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut et pulvinar nunc. Pellentesque fringilla mollis efficitur. Nullam venenatis commodo imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem sed turpis imperdiet eleifend sit amet id sapien.
+ EMBED LibreOffice.ChartDocument.1 
+:
+$
+rfHJLrt
+^
+HTXZ\­삂삂CJOJQJ	jU)0J:;B*phCJ@65OJQJjUU(:;B*phCJ@6&gt;*5OJQJ(:;B*phCJ@65]OJQJ(:;B*phCJ@65\OJQJ%:;B*phCJ@65OJQJ3 "$bnrtv!!!H"L",((B+/j028888899999湴Uj
+VUOJQJ	jU%:;B*phCJ@65OJQJ(:;B*phCJ@65\OJQJ%:;B*phCJ@65OJQJCJOJQJ(th{a
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F^]`hx$$a$1$^]`$d%d&amp;d'd$a$x
+`
+&amp;F^]`hx$$a$1$^]`$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd5~$$If\%	(p(474747474f4	$If$a$ $If$a$1$^]`$d%d&amp;d'd $If$a$1$^]`$d%d&amp;d'dJVXZ^X|$$If\%	(p(474747474f4 $If$a$1$^]`$d%d&amp;d'd	$If$a$^X7 $If$a$1$^]`$d%d&amp;d'd|$$If\%	(p(474747474f4	$If$a$ $If$a$1$^]`$d%d&amp;d'd "&amp;dpryX $If$a$1$^]`$d%d&amp;d'd|$$If\%	(p(474747474f4	$If$a$rtxyXyy $If$a$1$^]`$d%d&amp;d'd	$If$a$|$$If\%	(p(474747474f4!!!J"L".((D+ffffaff\f
+&amp;F
+&amp;F$a$1$^]`$d%d&amp;d'd|$$If\%	(p(474747474f4
+D+0l0288899 9
+&amp;F$a$1$^]`$d%d&amp;d'd	". A!n"n#n$n3P(20@=nD)M Ww l6},[ȏ&gt;o&lt;x[k\U&gt;ed~%F[$5uQVԔT`Q+%*n\rJ\I
+nAUUED(EE7ڍ ˽_ޝ3׃wrΜ9wLU	')=~Lē"('%S۰?{R]DnM7=٣~A_WM!~A%˝.lrz/ţ?O9ugmN\mGmalI5K{u]r/e߇G5WH1&gt;0Zr\.y'&gt;F^^FL~X_X3k+X3kɛX3kʘX3k=gò|bͬXe-ĚY렝sXւO35bU5`Y&gt;8=oX&gt;8֚m}bq,k'Zcͪ_kZ}5bq-r1~X\kg&amp;F,_#ZYЯc-sb377
+X?~*JU?ZJޭ4=1C.q'V譝?k"ƃ,8iƠ&gt;|`!x7B
+G&gt;cK+Z?f+%9C.nwH4ϹgrwCA{`!x7~W?Ϲgr7bl9k`:s,81?9C.n}CA{`!x7~K3A{`!r&lt;k_-ଷ\eMrJ_eI7;g3b3ZU&gt;S,-pGٕt\,|**̩/knƙI4o抢syPXsbj&gt;/ZQ4r֜X/HyV6SkNQDNF5^UA/UkN4?{VΉ_Q`0X=mNmϊ`X[`=:Ѷ=+gsam$ڶkE&gt;tX[`]DvFRFc휞mo{VT}zFC=a}z;ҷSϕO"(QJ_q,9.N.cz[ű\:8zN&gt;+%咗7Zo}
+~OψV7;7~\UXWM-&gt;[9im3|&amp;cEfmugXX;Ӷ}T.MS-\3/X?xFV:c;1JFIFHHXICC_PROFILEHLinomntrRGB XYZ 	1acspMSFTIEC sRGB-HP  cprtP3desclwtptbkptrXYZgXYZ,bXYZ@dmndTpdmddvuedLview$lumimeas$tech0rTRC&lt;gTRC&lt;bTRC&lt;textCopyright (c) 1998 Hewlett-Packard CompanydescsRGB IEC61966-2.1sRGB IEC61966-2.1XYZ QXYZ XYZ o8XYZ bXYZ $descIEC http://www.iec.chIEC http://www.iec.chdesc.IEC 61966-2.1 Default RGB colour space - sRGB.IEC 61966-2.1 Default RGB colour space - sRGBdesc,Reference Viewing Condition in IEC61966-2.1,Reference Viewing Condition in IEC61966-2.1view_.\XYZ L	VPWmeassig CRT curv
+#(-27;@EJOTY^chmrw|
+%+28&gt;ELRY`gnu|&amp;/8AKT]gqz!-8COZfr~ -;HUcq~
++:IXgw'7HYj{+=Oat2FZn		%	:	O	d	y						
+'
+=
+T
+j
+"9Qi*C\u
+&amp;
+@
+Z
+t
+.Id	%A^z	&amp;Ca~1Om&amp;Ed#Cc'Ij4Vx&amp;IlAe@e Ek*Qw;c*R{Gp@j&gt;i  A l   !!H!u!!!"'"U"""#
+#8#f###$$M$|$$%	%8%h%%%&amp;'&amp;W&amp;&amp;&amp;''I'z''(
+(?(q(())8)k))**5*h**++6+i++,,9,n,,--A-v--..L.../$/Z///050l0011J1112*2c223
+3F3334+4e4455M555676r667$7`7788P8899B999:6:t::;-;k;;&lt;'&lt;e&lt;&lt;="=a==&gt; &gt;`&gt;&gt;?!?a??@#@d@@A)AjAAB0BrBBC:C}CDDGDDEEUEEF"FgFFG5G{GHHKHHIIcIIJ7J}JKKSKKL*LrLMMJMMN%NnNOOIOOP'PqPQQPQQR1R|RSS_SSTBTTU(UuUVV\VVWDWWX/X}XYYiYZZVZZ[E[[\5\\]']x]^^l^__a_``W``aOaabIbbcCccd@dde=eef=ffg=ggh?hhiCiijHjjkOkklWlmm`mnnknooxop+ppq:qqrKrss]sttptu(uuv&gt;vvwVwxxnxy*yyzFz{{c{|!||}A}~~b~#G
+k͂0WGrׇ;iΉ3dʋ0cʍ</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>02322ecf-25a1-4fa0-8ec3-8170732b158b</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>--- Page 1 ---
+Sample Service Agreement
+This Service Agreement is entered into between Company A and Company B.
+Effective Date: January 1, 2025
+Expiration Date: December 31, 2025
+Payment Clause: Company B shall pay Company A $10,000 per month.
+Confidentiality Clause: Both parties agree to keep confidential information private.
+Termination Clause: Either party may terminate with 30 days written notice.
+Governing Law: State of California.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>a4a4156e-13d5-4287-b21b-312a8cf8f963</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>file-sample_100kB.doc</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ࡱ;		
+ !"#$%&amp;'()*+,-./0123456789:;&lt;=&gt;?@ABCDEFGHIJKLMNOPQRSTUVWXYZ[\]^_`abcdefghijklmnopqrstuvwxyz{|}~Root Entry	
+ !"#$%&amp;'()*+,-./0123456789:;&lt;=&gt;?@ABCE
+	FMicrosoft Word-Dokument
+MSWordDocWord.Document.89qDyKyKNhttps://products.office.com/en-us/wordOh+'0
+px	
+[ZZNormal1$*$3B*OJQJCJmH	sH	KHPJnHtH^JaJ_H9N!2N	Heading 1@&amp;
+&amp;F
+&amp;FxCJ$5aJ$\N!2N	Heading 2@&amp;
+&amp;F
+&amp;FxCJ 5aJ \X!2X	Heading 3@&amp;
+&amp;F
+&amp;FxB*phCJ5aJ\..BulletsOJQJPJ^JJUJ
+Internet Link B*	phmHsH&gt;*nHtH_HZVZVisited Internet Link B*
+phmHsH&gt;*nHtH_HF2FHeading
+x$OJ	QJ	CJPJ^JaJ4B24	Text Bodyd  /1B List^J
+@"R@Caption
+xx$CJ6^J
+aJ]&amp;b&amp;Index$^J
+&lt;r&lt;
+Quotations^7]7`2&gt;!22Title$a$CJ85aJ8\:J!2:Subtitle$a$&lt;xCJ$aJ$44Table Contents$*+*+P9^rD+ 9 !"#$%&amp;'%9dX%'+:X"$D)M Ww v$PR$V:c;1U@|(	
+NA?C"
+NA?C"&lt;
+Cb:r V
+T%(T^`P^`^8`08^`^X`X^`^x`x^``^`^`OJQJ^J^8`8OJQJ^J%^`OJQJ^J%^`OJQJ^J^p`pOJQJ^J%^	`	OJQJ^J%^@`@OJQJ^J^`OJQJ^J%^`OJQJ^J%P
+GTimes New Roman5Symbol3&amp;ArialiLiberation SerifTimes New Roman?&amp;DejaVu SansG
+Open SansArialODroid Sans Fallback9FreeSans_OpenSymbolArial Unicode MSS&amp;Liberation SansArial9$FreeSans5Symbol_OpenSymbolArial Unicode MSBhXg((((' 0 0
+0@@@B.o@
+
+;OBq*sLibreOffice.ChartDocument.1Embedded Object},[PKYKl((mimetypeapplication/vnd.oasis.openM 	0 9Caolan80	aNd+	FFLB
+!b-@6F8 :,~
+!Lorem ipsum 
+Lorem ipsum dolor sit amet, consectetur adipiscing elit. Nunc ac faucibus odio. 
+Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis, vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum, ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus.
+Maecenas non lorem quis tellus placerat varius. 
+Nulla facilisi. 
+Aenean congue fringilla justo ut aliquam. 
+ HYPERLINK "https://products.office.com/en-us/word"Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante sagittis. 
+Morbi viverra semper lorem nec molestie. 
+Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel, ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci maximus ultricies. 
+Cras fringilla ipsum magna, in fringilla dui commodo a.
+Lorem ipsumLorem ipsumLorem ipsum1In eleifend velit vitae libero sollicitudin euismod.Lorem2Cras fringilla ipsum magna, in fringilla dui commodo a.Ipsum3Aliquam erat volutpat. Lorem4Fusce vitae vestibulum velit. Lorem5Etiam vehicula luctus fermentum.Ipsum
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui. Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam, pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut et pulvinar nunc. Pellentesque fringilla mollis efficitur. Nullam venenatis commodo imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem sed turpis imperdiet eleifend sit amet id sapien.
+Lorem ipsum dolor sit amet, consectetur adipiscing elit. 
+Nunc ac faucibus odio. Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis, vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum, ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus. 
+Maecenas non lorem quis tellus placerat varius. Nulla facilisi. Aenean congue fringilla justo ut aliquam. Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante sagittis. Morbi viverra semper lorem nec molestie. Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel, ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. 
+Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci maximus ultricies. Cras fringilla ipsum magna, in fringilla dui commodo a.
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui. Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam, pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut et pulvinar nunc. Pellentesque fringilla mollis efficitur. Nullam venenatis commodo imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem sed turpis imperdiet eleifend sit amet id sapien.
+ EMBED LibreOffice.ChartDocument.1 
+:
+$
+rfHJLrt
+^
+HTXZ\­삂삂CJOJQJ	jU)0J:;B*phCJ@65OJQJjUU(:;B*phCJ@6&gt;*5OJQJ(:;B*phCJ@65]OJQJ(:;B*phCJ@65\OJQJ%:;B*phCJ@65OJQJ3 "$bnrtv!!!H"L",((B+/j028888899999湴Uj
+VUOJQJ	jU%:;B*phCJ@65OJQJ(:;B*phCJ@65\OJQJ%:;B*phCJ@65OJQJCJOJQJ(th{a
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F^]`hx$$a$1$^]`$d%d&amp;d'd$a$x
+`
+&amp;F^]`hx$$a$1$^]`$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd5~$$If\%	(p(474747474f4	$If$a$ $If$a$1$^]`$d%d&amp;d'd $If$a$1$^]`$d%d&amp;d'dJVXZ^X|$$If\%	(p(474747474f4 $If$a$1$^]`$d%d&amp;d'd	$If$a$^X7 $If$a$1$^]`$d%d&amp;d'd|$$If\%	(p(474747474f4	$If$a$ $If$a$1$^]`$d%d&amp;d'd "&amp;dpryX $If$a$1$^]`$d%d&amp;d'd|$$If\%	(p(474747474f4	$If$a$rtxyXyy $If$a$1$^]`$d%d&amp;d'd	$If$a$|$$If\%	(p(474747474f4!!!J"L".((D+ffffaff\f
+&amp;F
+&amp;F$a$1$^]`$d%d&amp;d'd|$$If\%	(p(474747474f4
+D+0l0288899 9
+&amp;F$a$1$^]`$d%d&amp;d'd	". A!n"n#n$n3P(20@=nD)M Ww l6},[ȏ&gt;o&lt;x[k\U&gt;ed~%F[$5uQVԔT`Q+%*n\rJ\I
+nAUUED(EE7ڍ ˽_ޝ3׃wrΜ9wLU	')=~Lē"('%S۰?{R]DnM7=٣~A_WM!~A%˝.lrz/ţ?O9ugmN\mGmalI5K{u]r/e߇G5WH1&gt;0Zr\.y'&gt;F^^FL~X_X3k+X3kɛX3kʘX3k=gò|bͬXe-ĚY렝sXւO35bU5`Y&gt;8=oX&gt;8֚m}bq,k'Zcͪ_kZ}5bq-r1~X\kg&amp;F,_#ZYЯc-sb377
+X?~*JU?ZJޭ4=1C.q'V譝?k"ƃ,8iƠ&gt;|`!x7B
+G&gt;cK+Z?f+%9C.nwH4ϹgrwCA{`!x7~W?Ϲgr7bl9k`:s,81?9C.n}CA{`!x7~K3A{`!r&lt;k_-ଷ\eMrJ_eI7;g3b3ZU&gt;S,-pGٕt\,|**̩/knƙI4o抢syPXsbj&gt;/ZQ4r֜X/HyV6SkNQDNF5^UA/UkN4?{VΉ_Q`0X=mNmϊ`X[`=:Ѷ=+gsam$ڶkE&gt;tX[`]DvFRFc휞mo{VT}zFC=a}z;ҷSϕO"(QJ_q,9.N.cz[ű\:8zN&gt;+%咗7Zo}
+~OψV7;7~\UXWM-&gt;[9im3|&amp;cEfmugXX;Ӷ}T.MS-\3/X?xFV:c;1JFIFHHXICC_PROFILEHLinomntrRGB XYZ 	1acspMSFTIEC sRGB-HP  cprtP3desclwtptbkptrXYZgXYZ,bXYZ@dmndTpdmddvuedLview$lumimeas$tech0rTRC&lt;gTRC&lt;bTRC&lt;textCopyright (c) 1998 Hewlett-Packard CompanydescsRGB IEC61966-2.1sRGB IEC61966-2.1XYZ QXYZ XYZ o8XYZ bXYZ $descIEC http://www.iec.chIEC http://www.iec.chdesc.IEC 61966-2.1 Default RGB colour space - sRGB.IEC 61966-2.1 Default RGB colour space - sRGBdesc,Reference Viewing Condition in IEC61966-2.1,Reference Viewing Condition in IEC61966-2.1view_.\XYZ L	VPWmeassig CRT curv
+#(-27;@EJOTY^chmrw|
+%+28&gt;ELRY`gnu|&amp;/8AKT]gqz!-8COZfr~ -;HUcq~
++:IXgw'7HYj{+=Oat2FZn		%	:	O	d	y						
+'
+=
+T
+j
+"9Qi*C\u
+&amp;
+@
+Z
+t
+.Id	%A^z	&amp;Ca~1Om&amp;Ed#Cc'Ij4Vx&amp;IlAe@e Ek*Qw;c*R{Gp@j&gt;i  A l   !!H!u!!!"'"U"""#
+#8#f###$$M$|$$%	%8%h%%%&amp;'&amp;W&amp;&amp;&amp;''I'z''(
+(?(q(())8)k))**5*h**++6+i++,,9,n,,--A-v--..L.../$/Z///050l0011J1112*2c223
+3F3334+4e4455M555676r667$7`7788P8899B999:6:t::;-;k;;&lt;'&lt;e&lt;&lt;="=a==&gt; &gt;`&gt;&gt;?!?a??@#@d@@A)AjAAB0BrBBC:C}CDDGDDEEUEEF"FgFFG5G{GHHKHHIIcIIJ7J}JKKSKKL*LrLMMJMMN%NnNOOIOOP'PqPQQPQQR1R|RSS_SSTBTTU(UuUVV\VVWDWWX/X}XYYiYZZVZZ[E[[\5\\]']x]^^l^__a_``W``aOaabIbbcCccd@dde=eef=ffg=ggh?hhiCiijHjjkOkklWlmm`mnnknooxop+ppq:qqrKrss]sttptu(uuv&gt;vvwVwxxnxy*yyzFz{{c{|!||}A}~~b~#G
+k͂0WGrׇ;iΉ3dʋ0cʍ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>9d53d74b-da2a-4072-8402-890806ece509</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>--- Page 1 ---
+Sample Service Agreement
+This Service Agreement is entered into between Company A and Company B.
+Effective Date: January 1, 2025
+Expiration Date: December 31, 2025
+Payment Clause: Company B shall pay Company A $10,000 per month.
+Confidentiality Clause: Both parties agree to keep confidential information private.
+Termination Clause: Either party may terminate with 30 days written notice.
+Governing Law: State of California.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>f5d109b6-8bdf-4364-bfa0-8d10c795291f</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>file-sample_100kB.doc</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ࡱ;		
+ !"#$%&amp;'()*+,-./0123456789:;&lt;=&gt;?@ABCDEFGHIJKLMNOPQRSTUVWXYZ[\]^_`abcdefghijklmnopqrstuvwxyz{|}~Root Entry	
+ !"#$%&amp;'()*+,-./0123456789:;&lt;=&gt;?@ABCE
+	FMicrosoft Word-Dokument
+MSWordDocWord.Document.89qDyKyKNhttps://products.office.com/en-us/wordOh+'0
+px	
+[ZZNormal1$*$3B*OJQJCJmH	sH	KHPJnHtH^JaJ_H9N!2N	Heading 1@&amp;
+&amp;F
+&amp;FxCJ$5aJ$\N!2N	Heading 2@&amp;
+&amp;F
+&amp;FxCJ 5aJ \X!2X	Heading 3@&amp;
+&amp;F
+&amp;FxB*phCJ5aJ\..BulletsOJQJPJ^JJUJ
+Internet Link B*	phmHsH&gt;*nHtH_HZVZVisited Internet Link B*
+phmHsH&gt;*nHtH_HF2FHeading
+x$OJ	QJ	CJPJ^JaJ4B24	Text Bodyd  /1B List^J
+@"R@Caption
+xx$CJ6^J
+aJ]&amp;b&amp;Index$^J
+&lt;r&lt;
+Quotations^7]7`2&gt;!22Title$a$CJ85aJ8\:J!2:Subtitle$a$&lt;xCJ$aJ$44Table Contents$*+*+P9^rD+ 9 !"#$%&amp;'%9dX%'+:X"$D)M Ww v$PR$V:c;1U@|(	
+NA?C"
+NA?C"&lt;
+Cb:r V
+T%(T^`P^`^8`08^`^X`X^`^x`x^``^`^`OJQJ^J^8`8OJQJ^J%^`OJQJ^J%^`OJQJ^J^p`pOJQJ^J%^	`	OJQJ^J%^@`@OJQJ^J^`OJQJ^J%^`OJQJ^J%P
+GTimes New Roman5Symbol3&amp;ArialiLiberation SerifTimes New Roman?&amp;DejaVu SansG
+Open SansArialODroid Sans Fallback9FreeSans_OpenSymbolArial Unicode MSS&amp;Liberation SansArial9$FreeSans5Symbol_OpenSymbolArial Unicode MSBhXg((((' 0 0
+0@@@B.o@
+
+;OBq*sLibreOffice.ChartDocument.1Embedded Object},[PKYKl((mimetypeapplication/vnd.oasis.openM 	0 9Caolan80	aNd+	FFLB
+!b-@6F8 :,~
+!Lorem ipsum 
+Lorem ipsum dolor sit amet, consectetur adipiscing elit. Nunc ac faucibus odio. 
+Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis, vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum, ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus.
+Maecenas non lorem quis tellus placerat varius. 
+Nulla facilisi. 
+Aenean congue fringilla justo ut aliquam. 
+ HYPERLINK "https://products.office.com/en-us/word"Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante sagittis. 
+Morbi viverra semper lorem nec molestie. 
+Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel, ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci maximus ultricies. 
+Cras fringilla ipsum magna, in fringilla dui commodo a.
+Lorem ipsumLorem ipsumLorem ipsum1In eleifend velit vitae libero sollicitudin euismod.Lorem2Cras fringilla ipsum magna, in fringilla dui commodo a.Ipsum3Aliquam erat volutpat. Lorem4Fusce vitae vestibulum velit. Lorem5Etiam vehicula luctus fermentum.Ipsum
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui. Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam, pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut et pulvinar nunc. Pellentesque fringilla mollis efficitur. Nullam venenatis commodo imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem sed turpis imperdiet eleifend sit amet id sapien.
+Lorem ipsum dolor sit amet, consectetur adipiscing elit. 
+Nunc ac faucibus odio. Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis, vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum, ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus. 
+Maecenas non lorem quis tellus placerat varius. Nulla facilisi. Aenean congue fringilla justo ut aliquam. Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante sagittis. Morbi viverra semper lorem nec molestie. Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel, ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. 
+Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci maximus ultricies. Cras fringilla ipsum magna, in fringilla dui commodo a.
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui. Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam, pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut et pulvinar nunc. Pellentesque fringilla mollis efficitur. Nullam venenatis commodo imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem sed turpis imperdiet eleifend sit amet id sapien.
+ EMBED LibreOffice.ChartDocument.1 
+:
+$
+rfHJLrt
+^
+HTXZ\­삂삂CJOJQJ	jU)0J:;B*phCJ@65OJQJjUU(:;B*phCJ@6&gt;*5OJQJ(:;B*phCJ@65]OJQJ(:;B*phCJ@65\OJQJ%:;B*phCJ@65OJQJ3 "$bnrtv!!!H"L",((B+/j028888899999湴Uj
+VUOJQJ	jU%:;B*phCJ@65OJQJ(:;B*phCJ@65\OJQJ%:;B*phCJ@65OJQJCJOJQJ(th{a
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F^]`hx$$a$1$^]`$d%d&amp;d'd$a$x
+`
+&amp;F^]`hx$$a$1$^]`$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd5~$$If\%	(p(474747474f4	$If$a$ $If$a$1$^]`$d%d&amp;d'd $If$a$1$^]`$d%d&amp;d'dJVXZ^X|$$If\%	(p(474747474f4 $If$a$1$^]`$d%d&amp;d'd	$If$a$^X7 $If$a$1$^]`$d%d&amp;d'd|$$If\%	(p(474747474f4	$If$a$ $If$a$1$^]`$d%d&amp;d'd "&amp;dpryX $If$a$1$^]`$d%d&amp;d'd|$$If\%	(p(474747474f4	$If$a$rtxyXyy $If$a$1$^]`$d%d&amp;d'd	$If$a$|$$If\%	(p(474747474f4!!!J"L".((D+ffffaff\f
+&amp;F
+&amp;F$a$1$^]`$d%d&amp;d'd|$$If\%	(p(474747474f4
+D+0l0288899 9
+&amp;F$a$1$^]`$d%d&amp;d'd	". A!n"n#n$n3P(20@=nD)M Ww l6},[ȏ&gt;o&lt;x[k\U&gt;ed~%F[$5uQVԔT`Q+%*n\rJ\I
+nAUUED(EE7ڍ ˽_ޝ3׃wrΜ9wLU	')=~Lē"('%S۰?{R]DnM7=٣~A_WM!~A%˝.lrz/ţ?O9ugmN\mGmalI5K{u]r/e߇G5WH1&gt;0Zr\.y'&gt;F^^FL~X_X3k+X3kɛX3kʘX3k=gò|bͬXe-ĚY렝sXւO35bU5`Y&gt;8=oX&gt;8֚m}bq,k'Zcͪ_kZ}5bq-r1~X\kg&amp;F,_#ZYЯc-sb377
+X?~*JU?ZJޭ4=1C.q'V譝?k"ƃ,8iƠ&gt;|`!x7B
+G&gt;cK+Z?f+%9C.nwH4ϹgrwCA{`!x7~W?Ϲgr7bl9k`:s,81?9C.n}CA{`!x7~K3A{`!r&lt;k_-ଷ\eMrJ_eI7;g3b3ZU&gt;S,-pGٕt\,|**̩/knƙI4o抢syPXsbj&gt;/ZQ4r֜X/HyV6SkNQDNF5^UA/UkN4?{VΉ_Q`0X=mNmϊ`X[`=:Ѷ=+gsam$ڶkE&gt;tX[`]DvFRFc휞mo{VT}zFC=a}z;ҷSϕO"(QJ_q,9.N.cz[ű\:8zN&gt;+%咗7Zo}
+~OψV7;7~\UXWM-&gt;[9im3|&amp;cEfmugXX;Ӷ}T.MS-\3/X?xFV:c;1JFIFHHXICC_PROFILEHLinomntrRGB XYZ 	1acspMSFTIEC sRGB-HP  cprtP3desclwtptbkptrXYZgXYZ,bXYZ@dmndTpdmddvuedLview$lumimeas$tech0rTRC&lt;gTRC&lt;bTRC&lt;textCopyright (c) 1998 Hewlett-Packard CompanydescsRGB IEC61966-2.1sRGB IEC61966-2.1XYZ QXYZ XYZ o8XYZ bXYZ $descIEC http://www.iec.chIEC http://www.iec.chdesc.IEC 61966-2.1 Default RGB colour space - sRGB.IEC 61966-2.1 Default RGB colour space - sRGBdesc,Reference Viewing Condition in IEC61966-2.1,Reference Viewing Condition in IEC61966-2.1view_.\XYZ L	VPWmeassig CRT curv
+#(-27;@EJOTY^chmrw|
+%+28&gt;ELRY`gnu|&amp;/8AKT]gqz!-8COZfr~ -;HUcq~
++:IXgw'7HYj{+=Oat2FZn		%	:	O	d	y						
+'
+=
+T
+j
+"9Qi*C\u
+&amp;
+@
+Z
+t
+.Id	%A^z	&amp;Ca~1Om&amp;Ed#Cc'Ij4Vx&amp;IlAe@e Ek*Qw;c*R{Gp@j&gt;i  A l   !!H!u!!!"'"U"""#
+#8#f###$$M$|$$%	%8%h%%%&amp;'&amp;W&amp;&amp;&amp;''I'z''(
+(?(q(())8)k))**5*h**++6+i++,,9,n,,--A-v--..L.../$/Z///050l0011J1112*2c223
+3F3334+4e4455M555676r667$7`7788P8899B999:6:t::;-;k;;&lt;'&lt;e&lt;&lt;="=a==&gt; &gt;`&gt;&gt;?!?a??@#@d@@A)AjAAB0BrBBC:C}CDDGDDEEUEEF"FgFFG5G{GHHKHHIIcIIJ7J}JKKSKKL*LrLMMJMMN%NnNOOIOOP'PqPQQPQQR1R|RSS_SSTBTTU(UuUVV\VVWDWWX/X}XYYiYZZVZZ[E[[\5\\]']x]^^l^__a_``W``aOaabIbbcCccd@dde=eef=ffg=ggh?hhiCiijHjjkOkklWlmm`mnnknooxop+ppq:qqrKrss]sttptu(uuv&gt;vvwVwxxnxy*yyzFz{{c{|!||}A}~~b~#G
+k͂0WGrׇ;iΉ3dʋ0cʍ</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>6882dc89-ec45-480e-9b40-68026dc5b421</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>--- Page 1 ---
+Sample Service Agreement
+This Service Agreement is entered into between Company A and Company B.
+Effective Date: January 1, 2025
+Expiration Date: December 31, 2025
+Payment Clause: Company B shall pay Company A $10,000 per month.
+Confidentiality Clause: Both parties agree to keep confidential information private.
+Termination Clause: Either party may terminate with 30 days written notice.
+Governing Law: State of California.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>df910248-91c5-45a6-b3d2-deb8d52c50e2</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>file-sample_100kB.doc</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ࡱ;		
+ !"#$%&amp;'()*+,-./0123456789:;&lt;=&gt;?@ABCDEFGHIJKLMNOPQRSTUVWXYZ[\]^_`abcdefghijklmnopqrstuvwxyz{|}~Root Entry	
+ !"#$%&amp;'()*+,-./0123456789:;&lt;=&gt;?@ABCE
+	FMicrosoft Word-Dokument
+MSWordDocWord.Document.89qDyKyKNhttps://products.office.com/en-us/wordOh+'0
+px	
+[ZZNormal1$*$3B*OJQJCJmH	sH	KHPJnHtH^JaJ_H9N!2N	Heading 1@&amp;
+&amp;F
+&amp;FxCJ$5aJ$\N!2N	Heading 2@&amp;
+&amp;F
+&amp;FxCJ 5aJ \X!2X	Heading 3@&amp;
+&amp;F
+&amp;FxB*phCJ5aJ\..BulletsOJQJPJ^JJUJ
+Internet Link B*	phmHsH&gt;*nHtH_HZVZVisited Internet Link B*
+phmHsH&gt;*nHtH_HF2FHeading
+x$OJ	QJ	CJPJ^JaJ4B24	Text Bodyd  /1B List^J
+@"R@Caption
+xx$CJ6^J
+aJ]&amp;b&amp;Index$^J
+&lt;r&lt;
+Quotations^7]7`2&gt;!22Title$a$CJ85aJ8\:J!2:Subtitle$a$&lt;xCJ$aJ$44Table Contents$*+*+P9^rD+ 9 !"#$%&amp;'%9dX%'+:X"$D)M Ww v$PR$V:c;1U@|(	
+NA?C"
+NA?C"&lt;
+Cb:r V
+T%(T^`P^`^8`08^`^X`X^`^x`x^``^`^`OJQJ^J^8`8OJQJ^J%^`OJQJ^J%^`OJQJ^J^p`pOJQJ^J%^	`	OJQJ^J%^@`@OJQJ^J^`OJQJ^J%^`OJQJ^J%P
+GTimes New Roman5Symbol3&amp;ArialiLiberation SerifTimes New Roman?&amp;DejaVu SansG
+Open SansArialODroid Sans Fallback9FreeSans_OpenSymbolArial Unicode MSS&amp;Liberation SansArial9$FreeSans5Symbol_OpenSymbolArial Unicode MSBhXg((((' 0 0
+0@@@B.o@
+
+;OBq*sLibreOffice.ChartDocument.1Embedded Object},[PKYKl((mimetypeapplication/vnd.oasis.openM 	0 9Caolan80	aNd+	FFLB
+!b-@6F8 :,~
+!Lorem ipsum 
+Lorem ipsum dolor sit amet, consectetur adipiscing elit. Nunc ac faucibus odio. 
+Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis, vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum, ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus.
+Maecenas non lorem quis tellus placerat varius. 
+Nulla facilisi. 
+Aenean congue fringilla justo ut aliquam. 
+ HYPERLINK "https://products.office.com/en-us/word"Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante sagittis. 
+Morbi viverra semper lorem nec molestie. 
+Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel, ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci maximus ultricies. 
+Cras fringilla ipsum magna, in fringilla dui commodo a.
+Lorem ipsumLorem ipsumLorem ipsum1In eleifend velit vitae libero sollicitudin euismod.Lorem2Cras fringilla ipsum magna, in fringilla dui commodo a.Ipsum3Aliquam erat volutpat. Lorem4Fusce vitae vestibulum velit. Lorem5Etiam vehicula luctus fermentum.Ipsum
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui. Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam, pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut et pulvinar nunc. Pellentesque fringilla mollis efficitur. Nullam venenatis commodo imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem sed turpis imperdiet eleifend sit amet id sapien.
+Lorem ipsum dolor sit amet, consectetur adipiscing elit. 
+Nunc ac faucibus odio. Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis, vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum, ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus. 
+Maecenas non lorem quis tellus placerat varius. Nulla facilisi. Aenean congue fringilla justo ut aliquam. Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante sagittis. Morbi viverra semper lorem nec molestie. Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel, ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. 
+Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci maximus ultricies. Cras fringilla ipsum magna, in fringilla dui commodo a.
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui. Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam, pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut et pulvinar nunc. Pellentesque fringilla mollis efficitur. Nullam venenatis commodo imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem sed turpis imperdiet eleifend sit amet id sapien.
+ EMBED LibreOffice.ChartDocument.1 
+:
+$
+rfHJLrt
+^
+HTXZ\­삂삂CJOJQJ	jU)0J:;B*phCJ@65OJQJjUU(:;B*phCJ@6&gt;*5OJQJ(:;B*phCJ@65]OJQJ(:;B*phCJ@65\OJQJ%:;B*phCJ@65OJQJ3 "$bnrtv!!!H"L",((B+/j028888899999湴Uj
+VUOJQJ	jU%:;B*phCJ@65OJQJ(:;B*phCJ@65\OJQJ%:;B*phCJ@65OJQJCJOJQJ(th{a
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F^]`hx$$a$1$^]`$d%d&amp;d'd$a$x
+`
+&amp;F^]`hx$$a$1$^]`$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd5~$$If\%	(p(474747474f4	$If$a$ $If$a$1$^]`$d%d&amp;d'd $If$a$1$^]`$d%d&amp;d'dJVXZ^X|$$If\%	(p(474747474f4 $If$a$1$^]`$d%d&amp;d'd	$If$a$^X7 $If$a$1$^]`$d%d&amp;d'd|$$If\%	(p(474747474f4	$If$a$ $If$a$1$^]`$d%d&amp;d'd "&amp;dpryX $If$a$1$^]`$d%d&amp;d'd|$$If\%	(p(474747474f4	$If$a$rtxyXyy $If$a$1$^]`$d%d&amp;d'd	$If$a$|$$If\%	(p(474747474f4!!!J"L".((D+ffffaff\f
+&amp;F
+&amp;F$a$1$^]`$d%d&amp;d'd|$$If\%	(p(474747474f4
+D+0l0288899 9
+&amp;F$a$1$^]`$d%d&amp;d'd	". A!n"n#n$n3P(20@=nD)M Ww l6},[ȏ&gt;o&lt;x[k\U&gt;ed~%F[$5uQVԔT`Q+%*n\rJ\I
+nAUUED(EE7ڍ ˽_ޝ3׃wrΜ9wLU	')=~Lē"('%S۰?{R]DnM7=٣~A_WM!~A%˝.lrz/ţ?O9ugmN\mGmalI5K{u]r/e߇G5WH1&gt;0Zr\.y'&gt;F^^FL~X_X3k+X3kɛX3kʘX3k=gò|bͬXe-ĚY렝sXւO35bU5`Y&gt;8=oX&gt;8֚m}bq,k'Zcͪ_kZ}5bq-r1~X\kg&amp;F,_#ZYЯc-sb377
+X?~*JU?ZJޭ4=1C.q'V譝?k"ƃ,8iƠ&gt;|`!x7B
+G&gt;cK+Z?f+%9C.nwH4ϹgrwCA{`!x7~W?Ϲgr7bl9k`:s,81?9C.n}CA{`!x7~K3A{`!r&lt;k_-ଷ\eMrJ_eI7;g3b3ZU&gt;S,-pGٕt\,|**̩/knƙI4o抢syPXsbj&gt;/ZQ4r֜X/HyV6SkNQDNF5^UA/UkN4?{VΉ_Q`0X=mNmϊ`X[`=:Ѷ=+gsam$ڶkE&gt;tX[`]DvFRFc휞mo{VT}zFC=a}z;ҷSϕO"(QJ_q,9.N.cz[ű\:8zN&gt;+%咗7Zo}
+~OψV7;7~\UXWM-&gt;[9im3|&amp;cEfmugXX;Ӷ}T.MS-\3/X?xFV:c;1JFIFHHXICC_PROFILEHLinomntrRGB XYZ 	1acspMSFTIEC sRGB-HP  cprtP3desclwtptbkptrXYZgXYZ,bXYZ@dmndTpdmddvuedLview$lumimeas$tech0rTRC&lt;gTRC&lt;bTRC&lt;textCopyright (c) 1998 Hewlett-Packard CompanydescsRGB IEC61966-2.1sRGB IEC61966-2.1XYZ QXYZ XYZ o8XYZ bXYZ $descIEC http://www.iec.chIEC http://www.iec.chdesc.IEC 61966-2.1 Default RGB colour space - sRGB.IEC 61966-2.1 Default RGB colour space - sRGBdesc,Reference Viewing Condition in IEC61966-2.1,Reference Viewing Condition in IEC61966-2.1view_.\XYZ L	VPWmeassig CRT curv
+#(-27;@EJOTY^chmrw|
+%+28&gt;ELRY`gnu|&amp;/8AKT]gqz!-8COZfr~ -;HUcq~
++:IXgw'7HYj{+=Oat2FZn		%	:	O	d	y						
+'
+=
+T
+j
+"9Qi*C\u
+&amp;
+@
+Z
+t
+.Id	%A^z	&amp;Ca~1Om&amp;Ed#Cc'Ij4Vx&amp;IlAe@e Ek*Qw;c*R{Gp@j&gt;i  A l   !!H!u!!!"'"U"""#
+#8#f###$$M$|$$%	%8%h%%%&amp;'&amp;W&amp;&amp;&amp;''I'z''(
+(?(q(())8)k))**5*h**++6+i++,,9,n,,--A-v--..L.../$/Z///050l0011J1112*2c223
+3F3334+4e4455M555676r667$7`7788P8899B999:6:t::;-;k;;&lt;'&lt;e&lt;&lt;="=a==&gt; &gt;`&gt;&gt;?!?a??@#@d@@A)AjAAB0BrBBC:C}CDDGDDEEUEEF"FgFFG5G{GHHKHHIIcIIJ7J}JKKSKKL*LrLMMJMMN%NnNOOIOOP'PqPQQPQQR1R|RSS_SSTBTTU(UuUVV\VVWDWWX/X}XYYiYZZVZZ[E[[\5\\]']x]^^l^__a_``W``aOaabIbbcCccd@dde=eef=ffg=ggh?hhiCiijHjjkOkklWlmm`mnnknooxop+ppq:qqrKrss]sttptu(uuv&gt;vvwVwxxnxy*yyzFz{{c{|!||}A}~~b~#G
+k͂0WGrׇ;iΉ3dʋ0cʍ</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>7f84a4f8-5947-4a69-9a74-08393b2a8c73</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>--- Page 1 ---
+Sample Service Agreement
+This Service Agreement is entered into between Company A and Company B.
+Effective Date: January 1, 2025
+Expiration Date: December 31, 2025
+Payment Clause: Company B shall pay Company A $10,000 per month.
+Confidentiality Clause: Both parties agree to keep confidential information private.
+Termination Clause: Either party may terminate with 30 days written notice.
+Governing Law: State of California.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>643394d8-6cae-42fd-b536-12046f1056d9</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>file-sample_100kB.doc</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ࡱ;		
+ !"#$%&amp;'()*+,-./0123456789:;&lt;=&gt;?@ABCDEFGHIJKLMNOPQRSTUVWXYZ[\]^_`abcdefghijklmnopqrstuvwxyz{|}~Root Entry	
+ !"#$%&amp;'()*+,-./0123456789:;&lt;=&gt;?@ABCE
+	FMicrosoft Word-Dokument
+MSWordDocWord.Document.89qDyKyKNhttps://products.office.com/en-us/wordOh+'0
+px	
+[ZZNormal1$*$3B*OJQJCJmH	sH	KHPJnHtH^JaJ_H9N!2N	Heading 1@&amp;
+&amp;F
+&amp;FxCJ$5aJ$\N!2N	Heading 2@&amp;
+&amp;F
+&amp;FxCJ 5aJ \X!2X	Heading 3@&amp;
+&amp;F
+&amp;FxB*phCJ5aJ\..BulletsOJQJPJ^JJUJ
+Internet Link B*	phmHsH&gt;*nHtH_HZVZVisited Internet Link B*
+phmHsH&gt;*nHtH_HF2FHeading
+x$OJ	QJ	CJPJ^JaJ4B24	Text Bodyd  /1B List^J
+@"R@Caption
+xx$CJ6^J
+aJ]&amp;b&amp;Index$^J
+&lt;r&lt;
+Quotations^7]7`2&gt;!22Title$a$CJ85aJ8\:J!2:Subtitle$a$&lt;xCJ$aJ$44Table Contents$*+*+P9^rD+ 9 !"#$%&amp;'%9dX%'+:X"$D)M Ww v$PR$V:c;1U@|(	
+NA?C"
+NA?C"&lt;
+Cb:r V
+T%(T^`P^`^8`08^`^X`X^`^x`x^``^`^`OJQJ^J^8`8OJQJ^J%^`OJQJ^J%^`OJQJ^J^p`pOJQJ^J%^	`	OJQJ^J%^@`@OJQJ^J^`OJQJ^J%^`OJQJ^J%P
+GTimes New Roman5Symbol3&amp;ArialiLiberation SerifTimes New Roman?&amp;DejaVu SansG
+Open SansArialODroid Sans Fallback9FreeSans_OpenSymbolArial Unicode MSS&amp;Liberation SansArial9$FreeSans5Symbol_OpenSymbolArial Unicode MSBhXg((((' 0 0
+0@@@B.o@
+
+;OBq*sLibreOffice.ChartDocument.1Embedded Object},[PKYKl((mimetypeapplication/vnd.oasis.openM 	0 9Caolan80	aNd+	FFLB
+!b-@6F8 :,~
+!Lorem ipsum 
+Lorem ipsum dolor sit amet, consectetur adipiscing elit. Nunc ac faucibus odio. 
+Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis, vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum, ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus.
+Maecenas non lorem quis tellus placerat varius. 
+Nulla facilisi. 
+Aenean congue fringilla justo ut aliquam. 
+ HYPERLINK "https://products.office.com/en-us/word"Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante sagittis. 
+Morbi viverra semper lorem nec molestie. 
+Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel, ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci maximus ultricies. 
+Cras fringilla ipsum magna, in fringilla dui commodo a.
+Lorem ipsumLorem ipsumLorem ipsum1In eleifend velit vitae libero sollicitudin euismod.Lorem2Cras fringilla ipsum magna, in fringilla dui commodo a.Ipsum3Aliquam erat volutpat. Lorem4Fusce vitae vestibulum velit. Lorem5Etiam vehicula luctus fermentum.Ipsum
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui. Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam, pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut et pulvinar nunc. Pellentesque fringilla mollis efficitur. Nullam venenatis commodo imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem sed turpis imperdiet eleifend sit amet id sapien.
+Lorem ipsum dolor sit amet, consectetur adipiscing elit. 
+Nunc ac faucibus odio. Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis, vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum, ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus. 
+Maecenas non lorem quis tellus placerat varius. Nulla facilisi. Aenean congue fringilla justo ut aliquam. Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante sagittis. Morbi viverra semper lorem nec molestie. Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel, ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. 
+Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci maximus ultricies. Cras fringilla ipsum magna, in fringilla dui commodo a.
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui. Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam, pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut et pulvinar nunc. Pellentesque fringilla mollis efficitur. Nullam venenatis commodo imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem sed turpis imperdiet eleifend sit amet id sapien.
+ EMBED LibreOffice.ChartDocument.1 
+:
+$
+rfHJLrt
+^
+HTXZ\­삂삂CJOJQJ	jU)0J:;B*phCJ@65OJQJjUU(:;B*phCJ@6&gt;*5OJQJ(:;B*phCJ@65]OJQJ(:;B*phCJ@65\OJQJ%:;B*phCJ@65OJQJ3 "$bnrtv!!!H"L",((B+/j028888899999湴Uj
+VUOJQJ	jU%:;B*phCJ@65OJQJ(:;B*phCJ@65\OJQJ%:;B*phCJ@65OJQJCJOJQJ(th{a
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F^]`hx$$a$1$^]`$d%d&amp;d'd$a$x
+`
+&amp;F^]`hx$$a$1$^]`$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd5~$$If\%	(p(474747474f4	$If$a$ $If$a$1$^]`$d%d&amp;d'd $If$a$1$^]`$d%d&amp;d'dJVXZ^X|$$If\%	(p(474747474f4 $If$a$1$^]`$d%d&amp;d'd	$If$a$^X7 $If$a$1$^]`$d%d&amp;d'd|$$If\%	(p(474747474f4	$If$a$ $If$a$1$^]`$d%d&amp;d'd "&amp;dpryX $If$a$1$^]`$d%d&amp;d'd|$$If\%	(p(474747474f4	$If$a$rtxyXyy $If$a$1$^]`$d%d&amp;d'd	$If$a$|$$If\%	(p(474747474f4!!!J"L".((D+ffffaff\f
+&amp;F
+&amp;F$a$1$^]`$d%d&amp;d'd|$$If\%	(p(474747474f4
+D+0l0288899 9
+&amp;F$a$1$^]`$d%d&amp;d'd	". A!n"n#n$n3P(20@=nD)M Ww l6},[ȏ&gt;o&lt;x[k\U&gt;ed~%F[$5uQVԔT`Q+%*n\rJ\I
+nAUUED(EE7ڍ ˽_ޝ3׃wrΜ9wLU	')=~Lē"('%S۰?{R]DnM7=٣~A_WM!~A%˝.lrz/ţ?O9ugmN\mGmalI5K{u]r/e߇G5WH1&gt;0Zr\.y'&gt;F^^FL~X_X3k+X3kɛX3kʘX3k=gò|bͬXe-ĚY렝sXւO35bU5`Y&gt;8=oX&gt;8֚m}bq,k'Zcͪ_kZ}5bq-r1~X\kg&amp;F,_#ZYЯc-sb377
+X?~*JU?ZJޭ4=1C.q'V譝?k"ƃ,8iƠ&gt;|`!x7B
+G&gt;cK+Z?f+%9C.nwH4ϹgrwCA{`!x7~W?Ϲgr7bl9k`:s,81?9C.n}CA{`!x7~K3A{`!r&lt;k_-ଷ\eMrJ_eI7;g3b3ZU&gt;S,-pGٕt\,|**̩/knƙI4o抢syPXsbj&gt;/ZQ4r֜X/HyV6SkNQDNF5^UA/UkN4?{VΉ_Q`0X=mNmϊ`X[`=:Ѷ=+gsam$ڶkE&gt;tX[`]DvFRFc휞mo{VT}zFC=a}z;ҷSϕO"(QJ_q,9.N.cz[ű\:8zN&gt;+%咗7Zo}
+~OψV7;7~\UXWM-&gt;[9im3|&amp;cEfmugXX;Ӷ}T.MS-\3/X?xFV:c;1JFIFHHXICC_PROFILEHLinomntrRGB XYZ 	1acspMSFTIEC sRGB-HP  cprtP3desclwtptbkptrXYZgXYZ,bXYZ@dmndTpdmddvuedLview$lumimeas$tech0rTRC&lt;gTRC&lt;bTRC&lt;textCopyright (c) 1998 Hewlett-Packard CompanydescsRGB IEC61966-2.1sRGB IEC61966-2.1XYZ QXYZ XYZ o8XYZ bXYZ $descIEC http://www.iec.chIEC http://www.iec.chdesc.IEC 61966-2.1 Default RGB colour space - sRGB.IEC 61966-2.1 Default RGB colour space - sRGBdesc,Reference Viewing Condition in IEC61966-2.1,Reference Viewing Condition in IEC61966-2.1view_.\XYZ L	VPWmeassig CRT curv
+#(-27;@EJOTY^chmrw|
+%+28&gt;ELRY`gnu|&amp;/8AKT]gqz!-8COZfr~ -;HUcq~
++:IXgw'7HYj{+=Oat2FZn		%	:	O	d	y						
+'
+=
+T
+j
+"9Qi*C\u
+&amp;
+@
+Z
+t
+.Id	%A^z	&amp;Ca~1Om&amp;Ed#Cc'Ij4Vx&amp;IlAe@e Ek*Qw;c*R{Gp@j&gt;i  A l   !!H!u!!!"'"U"""#
+#8#f###$$M$|$$%	%8%h%%%&amp;'&amp;W&amp;&amp;&amp;''I'z''(
+(?(q(())8)k))**5*h**++6+i++,,9,n,,--A-v--..L.../$/Z///050l0011J1112*2c223
+3F3334+4e4455M555676r667$7`7788P8899B999:6:t::;-;k;;&lt;'&lt;e&lt;&lt;="=a==&gt; &gt;`&gt;&gt;?!?a??@#@d@@A)AjAAB0BrBBC:C}CDDGDDEEUEEF"FgFFG5G{GHHKHHIIcIIJ7J}JKKSKKL*LrLMMJMMN%NnNOOIOOP'PqPQQPQQR1R|RSS_SSTBTTU(UuUVV\VVWDWWX/X}XYYiYZZVZZ[E[[\5\\]']x]^^l^__a_``W``aOaabIbbcCccd@dde=eef=ffg=ggh?hhiCiijHjjkOkklWlmm`mnnknooxop+ppq:qqrKrss]sttptu(uuv&gt;vvwVwxxnxy*yyzFz{{c{|!||}A}~~b~#G
+k͂0WGrׇ;iΉ3dʋ0cʍ</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>04bf9fd3-6cd0-4a73-a15e-ad4fc525ae8d</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>sample_contract.pdf</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>--- Page 1 ---
+Sample Service Agreement
+This Service Agreement is entered into between Company A and Company B.
+Effective Date: January 1, 2025
+Expiration Date: December 31, 2025
+Payment Clause: Company B shall pay Company A $10,000 per month.
+Confidentiality Clause: Both parties agree to keep confidential information private.
+Termination Clause: Either party may terminate with 30 days written notice.
+Governing Law: State of California.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>cbf7f90a-4c4a-4844-ac98-c9c970fdaf57</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>file-sample_100kB.doc</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ࡱ;		
+ !"#$%&amp;'()*+,-./0123456789:;&lt;=&gt;?@ABCDEFGHIJKLMNOPQRSTUVWXYZ[\]^_`abcdefghijklmnopqrstuvwxyz{|}~Root Entry	
+ !"#$%&amp;'()*+,-./0123456789:;&lt;=&gt;?@ABCE
+	FMicrosoft Word-Dokument
+MSWordDocWord.Document.89qDyKyKNhttps://products.office.com/en-us/wordOh+'0
+px	
+[ZZNormal1$*$3B*OJQJCJmH	sH	KHPJnHtH^JaJ_H9N!2N	Heading 1@&amp;
+&amp;F
+&amp;FxCJ$5aJ$\N!2N	Heading 2@&amp;
+&amp;F
+&amp;FxCJ 5aJ \X!2X	Heading 3@&amp;
+&amp;F
+&amp;FxB*phCJ5aJ\..BulletsOJQJPJ^JJUJ
+Internet Link B*	phmHsH&gt;*nHtH_HZVZVisited Internet Link B*
+phmHsH&gt;*nHtH_HF2FHeading
+x$OJ	QJ	CJPJ^JaJ4B24	Text Bodyd  /1B List^J
+@"R@Caption
+xx$CJ6^J
+aJ]&amp;b&amp;Index$^J
+&lt;r&lt;
+Quotations^7]7`2&gt;!22Title$a$CJ85aJ8\:J!2:Subtitle$a$&lt;xCJ$aJ$44Table Contents$*+*+P9^rD+ 9 !"#$%&amp;'%9dX%'+:X"$D)M Ww v$PR$V:c;1U@|(	
+NA?C"
+NA?C"&lt;
+Cb:r V
+T%(T^`P^`^8`08^`^X`X^`^x`x^``^`^`OJQJ^J^8`8OJQJ^J%^`OJQJ^J%^`OJQJ^J^p`pOJQJ^J%^	`	OJQJ^J%^@`@OJQJ^J^`OJQJ^J%^`OJQJ^J%P
+GTimes New Roman5Symbol3&amp;ArialiLiberation SerifTimes New Roman?&amp;DejaVu SansG
+Open SansArialODroid Sans Fallback9FreeSans_OpenSymbolArial Unicode MSS&amp;Liberation SansArial9$FreeSans5Symbol_OpenSymbolArial Unicode MSBhXg((((' 0 0
+0@@@B.o@
+
+;OBq*sLibreOffice.ChartDocument.1Embedded Object},[PKYKl((mimetypeapplication/vnd.oasis.openM 	0 9Caolan80	aNd+	FFLB
+!b-@6F8 :,~
+!Lorem ipsum 
+Lorem ipsum dolor sit amet, consectetur adipiscing elit. Nunc ac faucibus odio. 
+Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis, vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum, ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus.
+Maecenas non lorem quis tellus placerat varius. 
+Nulla facilisi. 
+Aenean congue fringilla justo ut aliquam. 
+ HYPERLINK "https://products.office.com/en-us/word"Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante sagittis. 
+Morbi viverra semper lorem nec molestie. 
+Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel, ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci maximus ultricies. 
+Cras fringilla ipsum magna, in fringilla dui commodo a.
+Lorem ipsumLorem ipsumLorem ipsum1In eleifend velit vitae libero sollicitudin euismod.Lorem2Cras fringilla ipsum magna, in fringilla dui commodo a.Ipsum3Aliquam erat volutpat. Lorem4Fusce vitae vestibulum velit. Lorem5Etiam vehicula luctus fermentum.Ipsum
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui. Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam, pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut et pulvinar nunc. Pellentesque fringilla mollis efficitur. Nullam venenatis commodo imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem sed turpis imperdiet eleifend sit amet id sapien.
+Lorem ipsum dolor sit amet, consectetur adipiscing elit. 
+Nunc ac faucibus odio. Vestibulum neque massa, scelerisque sit amet ligula eu, congue molestie mi. Praesent ut varius sem. Nullam at porttitor arcu, nec lacinia nisi. Ut ac dolor vitae odio interdum condimentum. Vivamus dapibus sodales ex, vitae malesuada ipsum cursus convallis. Maecenas sed egestas nulla, ac condimentum orci. Mauris diam felis, vulputate ac suscipit et, iaculis non est. Curabitur semper arcu ac ligula semper, nec luctus nisl blandit. Integer lacinia ante ac libero lobortis imperdiet. Nullam mollis convallis ipsum, ac accumsan nunc vehicula vitae. Nulla eget justo in felis tristique fringilla. Morbi sit amet tortor quis risus auctor condimentum. Morbi in ullamcorper elit. Nulla iaculis tellus sit amet mauris tempus fringilla.
+Maecenas mauris lectus, lobortis et purus mattis, blandit dictum tellus. 
+Maecenas non lorem quis tellus placerat varius. Nulla facilisi. Aenean congue fringilla justo ut aliquam. Mauris id ex erat. Nunc vulputate neque vitae justo facilisis, non condimentum ante sagittis. Morbi viverra semper lorem nec molestie. Maecenas tincidunt est efficitur ligula euismod, sit amet ornare est vulputate.
+In non mauris justo. Duis vehicula mi vel mi pretium, a viverra erat efficitur. Cras aliquam est ac eros varius, id iaculis dui auctor. Duis pretium neque ligula, et pulvinar mi placerat et. Nulla nec nunc sit amet nunc posuere vestibulum. Ut id neque eget tortor mattis tristique. Donec ante est, blandit sit amet tristique vel, lacinia pulvinar arcu. Pellentesque scelerisque fermentum erat, id posuere justo pulvinar ut. Cras id eros sed enim aliquam lobortis. Sed lobortis nisl ut eros efficitur tincidunt. Cras justo mi, porttitor quis mattis vel, ultricies ut purus. Ut facilisis et lacus eu cursus.
+In eleifend velit vitae libero sollicitudin euismod. 
+Fusce vitae vestibulum velit. Pellentesque vulputate lectus quis pellentesque commodo. Aliquam erat volutpat. Vestibulum in egestas velit. Pellentesque fermentum nisl vitae fringilla venenatis. Etiam id mauris vitae orci maximus ultricies. Cras fringilla ipsum magna, in fringilla dui commodo a.
+Etiam vehicula luctus fermentum. In vel metus congue, pulvinar lectus vel, fermentum dui. Maecenas ante orci, egestas ut aliquet sit amet, sagittis a magna. Aliquam ante quam, pellentesque ut dignissim quis, laoreet eget est. Aliquam erat volutpat. Class aptent taciti sociosqu ad litora torquent per conubia nostra, per inceptos himenaeos. Ut ullamcorper justo sapien, in cursus libero viverra eget. Vivamus auctor imperdiet urna, at pulvinar leo posuere laoreet. Suspendisse neque nisl, fringilla at iaculis scelerisque, ornare vel dolor. Ut et pulvinar nunc. Pellentesque fringilla mollis efficitur. Nullam venenatis commodo imperdiet. Morbi velit neque, semper quis lorem quis, efficitur dignissim ipsum. Ut ac lorem sed turpis imperdiet eleifend sit amet id sapien.
+ EMBED LibreOffice.ChartDocument.1 
+:
+$
+rfHJLrt
+^
+HTXZ\­삂삂CJOJQJ	jU)0J:;B*phCJ@65OJQJjUU(:;B*phCJ@6&gt;*5OJQJ(:;B*phCJ@65]OJQJ(:;B*phCJ@65\OJQJ%:;B*phCJ@65OJQJ3 "$bnrtv!!!H"L",((B+/j028888899999湴Uj
+VUOJQJ	jU%:;B*phCJ@65OJQJ(:;B*phCJ@65\OJQJ%:;B*phCJ@65OJQJCJOJQJ(th{a
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F^]`hx$$a$1$^]`$d%d&amp;d'd$a$x
+`
+&amp;F^]`hx$$a$1$^]`$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd
+&amp;F$a$1$$d%d&amp;d'd5~$$If\%	(p(474747474f4	$If$a$ $If$a$1$^]`$d%d&amp;d'd $If$a$1$^]`$d%d&amp;d'dJVXZ^X|$$If\%	(p(474747474f4 $If$a$1$^]`$d%d&amp;d'd	$If$a$^X7 $If$a$1$^]`$d%d&amp;d'd|$$If\%	(p(474747474f4	$If$a$ $If$a$1$^]`$d%d&amp;d'd "&amp;dpryX $If$a$1$^]`$d%d&amp;d'd|$$If\%	(p(474747474f4	$If$a$rtxyXyy $If$a$1$^]`$d%d&amp;d'd	$If$a$|$$If\%	(p(474747474f4!!!J"L".((D+ffffaff\f
+&amp;F
+&amp;F$a$1$^]`$d%d&amp;d'd|$$If\%	(p(474747474f4
+D+0l0288899 9
+&amp;F$a$1$^]`$d%d&amp;d'd	". A!n"n#n$n3P(20@=nD)M Ww l6},[ȏ&gt;o&lt;x[k\U&gt;ed~%F[$5uQVԔT`Q+%*n\rJ\I
+nAUUED(EE7ڍ ˽_ޝ3׃wrΜ9wLU	')=~Lē"('%S۰?{R]DnM7=٣~A_WM!~A%˝.lrz/ţ?O9ugmN\mGmalI5K{u]r/e߇G5WH1&gt;0Zr\.y'&gt;F^^FL~X_X3k+X3kɛX3kʘX3k=gò|bͬXe-ĚY렝sXւO35bU5`Y&gt;8=oX&gt;8֚m}bq,k'Zcͪ_kZ}5bq-r1~X\kg&amp;F,_#ZYЯc-sb377
+X?~*JU?ZJޭ4=1C.q'V譝?k"ƃ,8iƠ&gt;|`!x7B
+G&gt;cK+Z?f+%9C.nwH4ϹgrwCA{`!x7~W?Ϲgr7bl9k`:s,81?9C.n}CA{`!x7~K3A{`!r&lt;k_-ଷ\eMrJ_eI7;g3b3ZU&gt;S,-pGٕt\,|**̩/knƙI4o抢syPXsbj&gt;/ZQ4r֜X/HyV6SkNQDNF5^UA/UkN4?{VΉ_Q`0X=mNmϊ`X[`=:Ѷ=+gsam$ڶkE&gt;tX[`]DvFRFc휞mo{VT}zFC=a}z;ҷSϕO"(QJ_q,9.N.cz[ű\:8zN&gt;+%咗7Zo}
+~OψV7;7~\UXWM-&gt;[9im3|&amp;cEfmugXX;Ӷ}T.MS-\3/X?xFV:c;1JFIFHHXICC_PROFILEHLinomntrRGB XYZ 	1acspMSFTIEC sRGB-HP  cprtP3desclwtptbkptrXYZgXYZ,bXYZ@dmndTpdmddvuedLview$lumimeas$tech0rTRC&lt;gTRC&lt;bTRC&lt;textCopyright (c) 1998 Hewlett-Packard CompanydescsRGB IEC61966-2.1sRGB IEC61966-2.1XYZ QXYZ XYZ o8XYZ bXYZ $descIEC http://www.iec.chIEC http://www.iec.chdesc.IEC 61966-2.1 Default RGB colour space - sRGB.IEC 61966-2.1 Default RGB colour space - sRGBdesc,Reference Viewing Condition in IEC61966-2.1,Reference Viewing Condition in IEC61966-2.1view_.\XYZ L	VPWmeassig CRT curv
+#(-27;@EJOTY^chmrw|
+%+28&gt;ELRY`gnu|&amp;/8AKT]gqz!-8COZfr~ -;HUcq~
++:IXgw'7HYj{+=Oat2FZn		%	:	O	d	y						
+'
+=
+T
+j
+"9Qi*C\u
+&amp;
+@
+Z
+t
+.Id	%A^z	&amp;Ca~1Om&amp;Ed#Cc'Ij4Vx&amp;IlAe@e Ek*Qw;c*R{Gp@j&gt;i  A l   !!H!u!!!"'"U"""#
+#8#f###$$M$|$$%	%8%h%%%&amp;'&amp;W&amp;&amp;&amp;''I'z''(
+(?(q(())8)k))**5*h**++6+i++,,9,n,,--A-v--..L.../$/Z///050l0011J1112*2c223
+3F3334+4e4455M555676r667$7`7788P8899B999:6:t::;-;k;;&lt;'&lt;e&lt;&lt;="=a==&gt; &gt;`&gt;&gt;?!?a??@#@d@@A)AjAAB0BrBBC:C}CDDGDDEEUEEF"FgFFG5G{GHHKHHIIcIIJ7J}JKKSKKL*LrLMMJMMN%NnNOOIOOP'PqPQQPQQR1R|RSS_SSTBTTU(UuUVV\VVWDWWX/X}XYYiYZZVZZ[E[[\5\\]']x]^^l^__a_``W``aOaabIbbcCccd@dde=eef=ffg=ggh?hhiCiijHjjkOkklWlmm`mnnknooxop+ppq:qqrKrss]sttptu(uuv&gt;vvwVwxxnxy*yyzFz{{c{|!||}A}~~b~#G
+k͂0WGrׇ;iΉ3dʋ0cʍ</t>
         </is>
       </c>
     </row>

</xml_diff>